<commit_message>
Test Plan 3, Test Report 3, Requirements, User Document
All above are added/updated
</commit_message>
<xml_diff>
--- a/Documents/project requirements spreadsheet.xlsx
+++ b/Documents/project requirements spreadsheet.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11110"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Files\Documents\__ School\CS 3300- Software Development\Project (Group 1)\Shattered-Protocols-Text-RPG\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/soapmac/Documents/GitHub/Shattered-Protocols-Text-RPG/Shattered Protocols/Shattered-Protocols-Text-RPG/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD6FA2E8-1760-406E-8B60-921C1221A390}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE46A757-6460-CC4F-9E9E-282D8A9E1569}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12696" xr2:uid="{CAB5D44A-E176-404C-B398-BEAD2D9E6884}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15800" xr2:uid="{CAB5D44A-E176-404C-B398-BEAD2D9E6884}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -979,44 +979,44 @@
     <xf numFmtId="16" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="14" fontId="13" fillId="7" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="14" fontId="13" fillId="7" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1361,120 +1361,120 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B900A37F-814E-4AF4-9047-E946E2A67EEB}">
   <dimension ref="A1:L166"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="15" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="15.44140625" style="6" customWidth="1"/>
+    <col min="1" max="1" width="15.5" style="6" customWidth="1"/>
     <col min="2" max="2" width="61.33203125" style="5" customWidth="1"/>
-    <col min="3" max="3" width="17.109375" style="6" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.1640625" style="6" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12.6640625" style="6" customWidth="1"/>
-    <col min="5" max="5" width="15.77734375" style="6" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.83203125" style="6" bestFit="1" customWidth="1"/>
     <col min="6" max="7" width="12.6640625" style="6" customWidth="1"/>
-    <col min="8" max="8" width="16.109375" style="6" customWidth="1"/>
+    <col min="8" max="8" width="16.1640625" style="6" customWidth="1"/>
     <col min="9" max="11" width="12.6640625" style="6" customWidth="1"/>
-    <col min="12" max="12" width="173.77734375" style="72" customWidth="1"/>
-    <col min="13" max="16384" width="9.109375" style="12"/>
+    <col min="12" max="12" width="173.83203125" style="72" customWidth="1"/>
+    <col min="13" max="16384" width="9.1640625" style="12"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" s="26" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="86" t="s">
+    <row r="1" spans="1:12" s="26" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="84" t="s">
         <v>85</v>
       </c>
-      <c r="B1" s="87"/>
+      <c r="B1" s="85"/>
       <c r="C1" s="24"/>
-      <c r="D1" s="92" t="s">
+      <c r="D1" s="90" t="s">
         <v>86</v>
       </c>
-      <c r="E1" s="92"/>
-      <c r="F1" s="92"/>
-      <c r="G1" s="92"/>
-      <c r="H1" s="92"/>
-      <c r="I1" s="92"/>
-      <c r="J1" s="92"/>
-      <c r="K1" s="92"/>
+      <c r="E1" s="90"/>
+      <c r="F1" s="90"/>
+      <c r="G1" s="90"/>
+      <c r="H1" s="90"/>
+      <c r="I1" s="90"/>
+      <c r="J1" s="90"/>
+      <c r="K1" s="90"/>
       <c r="L1" s="64"/>
     </row>
-    <row r="2" spans="1:12" s="26" customFormat="1" ht="18" x14ac:dyDescent="0.3">
-      <c r="A2" s="88" t="s">
+    <row r="2" spans="1:12" s="26" customFormat="1" ht="19" x14ac:dyDescent="0.2">
+      <c r="A2" s="86" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="89"/>
+      <c r="B2" s="87"/>
       <c r="C2" s="24"/>
-      <c r="D2" s="92"/>
-      <c r="E2" s="92"/>
-      <c r="F2" s="92"/>
-      <c r="G2" s="92"/>
-      <c r="H2" s="92"/>
-      <c r="I2" s="92"/>
-      <c r="J2" s="92"/>
-      <c r="K2" s="92"/>
+      <c r="D2" s="90"/>
+      <c r="E2" s="90"/>
+      <c r="F2" s="90"/>
+      <c r="G2" s="90"/>
+      <c r="H2" s="90"/>
+      <c r="I2" s="90"/>
+      <c r="J2" s="90"/>
+      <c r="K2" s="90"/>
       <c r="L2" s="65"/>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A3" s="41"/>
       <c r="B3" s="29"/>
       <c r="C3" s="12"/>
-      <c r="D3" s="92"/>
-      <c r="E3" s="92"/>
-      <c r="F3" s="92"/>
-      <c r="G3" s="92"/>
-      <c r="H3" s="92"/>
-      <c r="I3" s="92"/>
-      <c r="J3" s="92"/>
-      <c r="K3" s="92"/>
+      <c r="D3" s="90"/>
+      <c r="E3" s="90"/>
+      <c r="F3" s="90"/>
+      <c r="G3" s="90"/>
+      <c r="H3" s="90"/>
+      <c r="I3" s="90"/>
+      <c r="J3" s="90"/>
+      <c r="K3" s="90"/>
       <c r="L3" s="66"/>
     </row>
-    <row r="4" spans="1:12" s="7" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:12" s="7" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A4" s="42" t="s">
         <v>17</v>
       </c>
       <c r="B4" s="30" t="s">
         <v>39</v>
       </c>
-      <c r="D4" s="92"/>
-      <c r="E4" s="92"/>
-      <c r="F4" s="92"/>
-      <c r="G4" s="92"/>
-      <c r="H4" s="92"/>
-      <c r="I4" s="92"/>
-      <c r="J4" s="92"/>
-      <c r="K4" s="92"/>
+      <c r="D4" s="90"/>
+      <c r="E4" s="90"/>
+      <c r="F4" s="90"/>
+      <c r="G4" s="90"/>
+      <c r="H4" s="90"/>
+      <c r="I4" s="90"/>
+      <c r="J4" s="90"/>
+      <c r="K4" s="90"/>
       <c r="L4" s="67"/>
     </row>
-    <row r="5" spans="1:12" s="7" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:12" s="7" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A5" s="42" t="s">
         <v>18</v>
       </c>
       <c r="B5" s="30" t="s">
         <v>40</v>
       </c>
-      <c r="D5" s="92"/>
-      <c r="E5" s="92"/>
-      <c r="F5" s="92"/>
-      <c r="G5" s="92"/>
-      <c r="H5" s="92"/>
-      <c r="I5" s="92"/>
-      <c r="J5" s="92"/>
-      <c r="K5" s="92"/>
+      <c r="D5" s="90"/>
+      <c r="E5" s="90"/>
+      <c r="F5" s="90"/>
+      <c r="G5" s="90"/>
+      <c r="H5" s="90"/>
+      <c r="I5" s="90"/>
+      <c r="J5" s="90"/>
+      <c r="K5" s="90"/>
       <c r="L5" s="67"/>
     </row>
-    <row r="6" spans="1:12" s="7" customFormat="1" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:12" s="7" customFormat="1" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A6" s="43" t="s">
         <v>19</v>
       </c>
       <c r="B6" s="31" t="s">
         <v>84</v>
       </c>
-      <c r="D6" s="92"/>
-      <c r="E6" s="92"/>
-      <c r="F6" s="92"/>
-      <c r="G6" s="92"/>
-      <c r="H6" s="92"/>
-      <c r="I6" s="92"/>
-      <c r="J6" s="92"/>
-      <c r="K6" s="92"/>
+      <c r="D6" s="90"/>
+      <c r="E6" s="90"/>
+      <c r="F6" s="90"/>
+      <c r="G6" s="90"/>
+      <c r="H6" s="90"/>
+      <c r="I6" s="90"/>
+      <c r="J6" s="90"/>
+      <c r="K6" s="90"/>
       <c r="L6" s="68"/>
     </row>
-    <row r="7" spans="1:12" s="7" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:12" s="7" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A7" s="44"/>
       <c r="B7" s="2"/>
       <c r="C7" s="1"/>
@@ -1488,94 +1488,94 @@
       <c r="K7" s="1"/>
       <c r="L7" s="68"/>
     </row>
-    <row r="8" spans="1:12" s="7" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A8" s="85" t="s">
+    <row r="8" spans="1:12" s="7" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="83" t="s">
         <v>16</v>
       </c>
-      <c r="B8" s="85"/>
-      <c r="C8" s="85"/>
-      <c r="D8" s="85"/>
-      <c r="E8" s="85"/>
-      <c r="F8" s="85"/>
-      <c r="G8" s="85"/>
-      <c r="H8" s="85"/>
-      <c r="I8" s="85"/>
-      <c r="J8" s="85"/>
-      <c r="K8" s="85"/>
-      <c r="L8" s="85"/>
-    </row>
-    <row r="9" spans="1:12" s="7" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B8" s="83"/>
+      <c r="C8" s="83"/>
+      <c r="D8" s="83"/>
+      <c r="E8" s="83"/>
+      <c r="F8" s="83"/>
+      <c r="G8" s="83"/>
+      <c r="H8" s="83"/>
+      <c r="I8" s="83"/>
+      <c r="J8" s="83"/>
+      <c r="K8" s="83"/>
+      <c r="L8" s="83"/>
+    </row>
+    <row r="9" spans="1:12" s="7" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A9" s="1"/>
       <c r="B9" s="2"/>
-      <c r="C9" s="85" t="s">
+      <c r="C9" s="83" t="s">
         <v>15</v>
       </c>
-      <c r="D9" s="85"/>
-      <c r="E9" s="85"/>
-      <c r="F9" s="85"/>
+      <c r="D9" s="83"/>
+      <c r="E9" s="83"/>
+      <c r="F9" s="83"/>
       <c r="G9" s="1"/>
-      <c r="H9" s="85" t="s">
+      <c r="H9" s="83" t="s">
         <v>7</v>
       </c>
-      <c r="I9" s="85"/>
-      <c r="J9" s="85"/>
-      <c r="K9" s="85"/>
-      <c r="L9" s="93" t="s">
+      <c r="I9" s="83"/>
+      <c r="J9" s="83"/>
+      <c r="K9" s="83"/>
+      <c r="L9" s="91" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:12" s="7" customFormat="1" ht="15.45" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:12" s="7" customFormat="1" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1"/>
       <c r="B10" s="2"/>
-      <c r="C10" s="84" t="s">
+      <c r="C10" s="82" t="s">
         <v>20</v>
       </c>
       <c r="D10" s="1"/>
-      <c r="E10" s="84" t="s">
+      <c r="E10" s="82" t="s">
         <v>55</v>
       </c>
-      <c r="F10" s="84" t="s">
+      <c r="F10" s="82" t="s">
         <v>56</v>
       </c>
-      <c r="G10" s="84" t="s">
+      <c r="G10" s="82" t="s">
         <v>57</v>
       </c>
-      <c r="H10" s="84" t="s">
+      <c r="H10" s="82" t="s">
         <v>4</v>
       </c>
-      <c r="I10" s="84" t="s">
+      <c r="I10" s="82" t="s">
         <v>20</v>
       </c>
-      <c r="J10" s="84" t="s">
+      <c r="J10" s="82" t="s">
         <v>5</v>
       </c>
       <c r="K10" s="1"/>
-      <c r="L10" s="93"/>
-    </row>
-    <row r="11" spans="1:12" s="7" customFormat="1" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="L10" s="91"/>
+    </row>
+    <row r="11" spans="1:12" s="7" customFormat="1" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>1</v>
       </c>
       <c r="B11" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="C11" s="84"/>
+      <c r="C11" s="82"/>
       <c r="D11" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E11" s="84"/>
-      <c r="F11" s="84"/>
-      <c r="G11" s="84"/>
-      <c r="H11" s="84"/>
-      <c r="I11" s="84"/>
-      <c r="J11" s="84"/>
+      <c r="E11" s="82"/>
+      <c r="F11" s="82"/>
+      <c r="G11" s="82"/>
+      <c r="H11" s="82"/>
+      <c r="I11" s="82"/>
+      <c r="J11" s="82"/>
       <c r="K11" s="25" t="s">
         <v>6</v>
       </c>
-      <c r="L11" s="93"/>
-    </row>
-    <row r="12" spans="1:12" s="55" customFormat="1" ht="45.6" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="90" t="s">
+      <c r="L11" s="91"/>
+    </row>
+    <row r="12" spans="1:12" s="55" customFormat="1" ht="52" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="88" t="s">
         <v>38</v>
       </c>
       <c r="B12" s="52"/>
@@ -1600,8 +1600,8 @@
       </c>
       <c r="L12" s="69"/>
     </row>
-    <row r="13" spans="1:12" s="3" customFormat="1" ht="61.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="91"/>
+    <row r="13" spans="1:12" s="3" customFormat="1" ht="61.5" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="89"/>
       <c r="B13" s="8"/>
       <c r="C13" s="10"/>
       <c r="D13" s="10" t="s">
@@ -1620,7 +1620,7 @@
       <c r="K13" s="10"/>
       <c r="L13" s="70"/>
     </row>
-    <row r="14" spans="1:12" s="21" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:12" s="21" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A14" s="45">
         <v>0</v>
       </c>
@@ -1651,7 +1651,7 @@
       <c r="K14" s="19"/>
       <c r="L14" s="71"/>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A15" s="46">
         <f>A14+1</f>
         <v>1</v>
@@ -1676,7 +1676,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A16" s="46">
         <f t="shared" ref="A16:A32" si="0">A15+1</f>
         <v>2</v>
@@ -1701,7 +1701,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="17" spans="1:12" ht="15.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:12" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A17" s="46">
         <f t="shared" si="0"/>
         <v>3</v>
@@ -1726,7 +1726,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A18" s="46">
         <f t="shared" si="0"/>
         <v>4</v>
@@ -1751,7 +1751,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A19" s="46">
         <f t="shared" si="0"/>
         <v>5</v>
@@ -1776,7 +1776,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A20" s="46">
         <f t="shared" si="0"/>
         <v>6</v>
@@ -1801,7 +1801,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A21" s="46">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -1826,7 +1826,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A22" s="46">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -1851,7 +1851,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A23" s="46">
         <f t="shared" si="0"/>
         <v>9</v>
@@ -1876,7 +1876,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="24" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A24" s="46">
         <f t="shared" si="0"/>
         <v>10</v>
@@ -1901,7 +1901,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A25" s="46">
         <f t="shared" si="0"/>
         <v>11</v>
@@ -1929,7 +1929,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A26" s="46">
         <f t="shared" si="0"/>
         <v>12</v>
@@ -1957,7 +1957,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A27" s="46">
         <f t="shared" si="0"/>
         <v>13</v>
@@ -1982,7 +1982,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A28" s="46">
         <f t="shared" si="0"/>
         <v>14</v>
@@ -2007,7 +2007,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A29" s="46">
         <f t="shared" si="0"/>
         <v>15</v>
@@ -2032,7 +2032,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A30" s="46">
         <f t="shared" si="0"/>
         <v>16</v>
@@ -2057,7 +2057,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="31" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="46">
         <f t="shared" si="0"/>
         <v>17</v>
@@ -2082,7 +2082,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="32" spans="1:12" s="14" customFormat="1" ht="15.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:12" s="14" customFormat="1" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A32" s="47">
         <f t="shared" si="0"/>
         <v>18</v>
@@ -2112,7 +2112,7 @@
       <c r="K32" s="10"/>
       <c r="L32" s="73"/>
     </row>
-    <row r="33" spans="1:12" s="17" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:12" s="17" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="48">
         <f>IF(D33=D32,A32+1,(D33*100))</f>
         <v>0</v>
@@ -2144,7 +2144,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A34" s="49">
         <f t="shared" ref="A34:A44" si="2">IF(D34=D33,A33+1,(D34*100))</f>
         <v>1</v>
@@ -2171,11 +2171,11 @@
       <c r="H34" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="L34" s="81" t="s">
+      <c r="L34" s="92" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A35" s="49">
         <f t="shared" si="2"/>
         <v>2</v>
@@ -2202,9 +2202,9 @@
       <c r="H35" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="L35" s="82"/>
-    </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="L35" s="93"/>
+    </row>
+    <row r="36" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A36" s="49">
         <f t="shared" si="2"/>
         <v>3</v>
@@ -2231,9 +2231,9 @@
       <c r="H36" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="L36" s="82"/>
-    </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="L36" s="93"/>
+    </row>
+    <row r="37" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A37" s="49">
         <f t="shared" si="2"/>
         <v>4</v>
@@ -2260,9 +2260,9 @@
       <c r="H37" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="L37" s="82"/>
-    </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="L37" s="93"/>
+    </row>
+    <row r="38" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A38" s="49">
         <f t="shared" si="2"/>
         <v>5</v>
@@ -2289,9 +2289,9 @@
       <c r="H38" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="L38" s="82"/>
-    </row>
-    <row r="39" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="L38" s="93"/>
+    </row>
+    <row r="39" spans="1:12" ht="32" x14ac:dyDescent="0.2">
       <c r="A39" s="49">
         <f t="shared" si="2"/>
         <v>6</v>
@@ -2322,7 +2322,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A40" s="49">
         <f t="shared" si="2"/>
         <v>7</v>
@@ -2353,7 +2353,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A41" s="49">
         <f t="shared" si="2"/>
         <v>8</v>
@@ -2384,7 +2384,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A42" s="49">
         <f t="shared" si="2"/>
         <v>9</v>
@@ -2415,7 +2415,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A43" s="49">
         <f t="shared" si="2"/>
         <v>10</v>
@@ -2446,7 +2446,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="44" spans="1:12" s="14" customFormat="1" ht="15.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:12" s="14" customFormat="1" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A44" s="50">
         <f t="shared" si="2"/>
         <v>11</v>
@@ -2480,7 +2480,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="45" spans="1:12" s="38" customFormat="1" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:12" s="38" customFormat="1" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A45" s="51">
         <f>IF(D45=D43,A43+1,(D45*100))</f>
         <v>100</v>
@@ -2509,7 +2509,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="46" spans="1:12" s="17" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:12" s="17" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="48">
         <f>IF(D46=D44,A44+1,(D46*100))</f>
         <v>100</v>
@@ -2537,7 +2537,7 @@
       <c r="K46" s="16"/>
       <c r="L46" s="78"/>
     </row>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A47" s="40">
         <f t="shared" ref="A47:A108" si="3">IF(B47="","",IF(D47=D46,A46+1,(D47*100)))</f>
         <v>101</v>
@@ -2565,7 +2565,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="48" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A48" s="49">
         <f t="shared" si="3"/>
         <v>102</v>
@@ -2593,7 +2593,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="49" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A49" s="49">
         <f t="shared" si="3"/>
         <v>103</v>
@@ -2625,7 +2625,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="50" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A50" s="49">
         <f t="shared" si="3"/>
         <v>104</v>
@@ -2653,7 +2653,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="51" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A51" s="49">
         <f t="shared" si="3"/>
         <v>105</v>
@@ -2681,7 +2681,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="52" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A52" s="40">
         <f>IF(B52="","",IF(D52=D51,A51+1,(D52*100)))</f>
         <v>106</v>
@@ -2709,7 +2709,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="53" spans="1:12" ht="19.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:12" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="40" t="s">
         <v>100</v>
       </c>
@@ -2736,7 +2736,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="54" spans="1:12" ht="19.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:12" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="40">
         <f>IF(B54="","",IF(D54=Sheet1!D53,Sheet1!A53+1,(D54*100)))</f>
         <v>110.00000000000001</v>
@@ -2765,7 +2765,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="55" spans="1:12" s="61" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:12" s="61" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="56">
         <f>IF(B55="","",IF(D55=D52,A52+1,(D55*100)))</f>
         <v>200</v>
@@ -2794,7 +2794,7 @@
       <c r="K55" s="58"/>
       <c r="L55" s="79"/>
     </row>
-    <row r="56" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A56" s="40">
         <f>IF(B56="","",IF(D56=D53,A53+1,(D56*100)))</f>
         <v>200</v>
@@ -2822,7 +2822,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="57" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A57" s="40">
         <f>IF(B57="","",IF(D57=D62,A62+1,(D57*100)))</f>
         <v>202</v>
@@ -2851,7 +2851,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="58" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A58" s="40">
         <f t="shared" si="3"/>
         <v>203</v>
@@ -2866,11 +2866,11 @@
         <f t="shared" ref="D58:D120" si="5">IF(B58="","",D57)</f>
         <v>2</v>
       </c>
-      <c r="E58" s="83" t="s">
+      <c r="E58" s="81" t="s">
         <v>112</v>
       </c>
-      <c r="F58" s="83"/>
-      <c r="G58" s="83"/>
+      <c r="F58" s="81"/>
+      <c r="G58" s="81"/>
       <c r="H58" s="6" t="s">
         <v>92</v>
       </c>
@@ -2878,7 +2878,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="59" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A59" s="40">
         <f t="shared" si="3"/>
         <v>204</v>
@@ -2907,7 +2907,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="60" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A60" s="40">
         <f>IF(B60="","",IF(D60=D65,A65+1,(D60*100)))</f>
         <v>207</v>
@@ -2933,7 +2933,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="61" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A61" s="40">
         <f>IF(B61="","",IF(D61=D60,A60+1,(D61*100)))</f>
         <v>208</v>
@@ -2959,7 +2959,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="62" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A62" s="40">
         <f>IF(B62="","",IF(D62=D56,A56+1,(D62*100)))</f>
         <v>201</v>
@@ -2973,11 +2973,11 @@
       <c r="D62" s="6">
         <v>2</v>
       </c>
-      <c r="E62" s="83" t="s">
+      <c r="E62" s="81" t="s">
         <v>78</v>
       </c>
-      <c r="F62" s="83"/>
-      <c r="G62" s="83"/>
+      <c r="F62" s="81"/>
+      <c r="G62" s="81"/>
       <c r="H62" s="6" t="s">
         <v>92</v>
       </c>
@@ -2985,7 +2985,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="63" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A63" s="40">
         <f>IF(B63="","",IF(D63=D61,A61+1,(D63*100)))</f>
         <v>209</v>
@@ -3000,16 +3000,16 @@
         <f>IF(B63="","",D61)</f>
         <v>2</v>
       </c>
-      <c r="E63" s="83" t="s">
+      <c r="E63" s="81" t="s">
         <v>78</v>
       </c>
-      <c r="F63" s="83"/>
-      <c r="G63" s="83"/>
+      <c r="F63" s="81"/>
+      <c r="G63" s="81"/>
       <c r="L63" s="72" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="64" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A64" s="40">
         <f>IF(B64="","",IF(D64=D59,A59+1,(D64*100)))</f>
         <v>205</v>
@@ -3024,13 +3024,13 @@
         <f>IF(B64="","",D59)</f>
         <v>2</v>
       </c>
-      <c r="E64" s="83" t="s">
+      <c r="E64" s="81" t="s">
         <v>78</v>
       </c>
-      <c r="F64" s="83"/>
-      <c r="G64" s="83"/>
-    </row>
-    <row r="65" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="F64" s="81"/>
+      <c r="G64" s="81"/>
+    </row>
+    <row r="65" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A65" s="40">
         <f>IF(B65="","",IF(D65=D64,A64+1,(D65*100)))</f>
         <v>206</v>
@@ -3045,16 +3045,16 @@
         <f>IF(B65="","",D64)</f>
         <v>2</v>
       </c>
-      <c r="E65" s="83" t="s">
+      <c r="E65" s="81" t="s">
         <v>112</v>
       </c>
-      <c r="F65" s="83"/>
-      <c r="G65" s="83"/>
+      <c r="F65" s="81"/>
+      <c r="G65" s="81"/>
       <c r="L65" s="72" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="66" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A66" s="40">
         <f>IF(B66="","",IF(D66=D63,A63+1,(D66*100)))</f>
         <v>210</v>
@@ -3080,7 +3080,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="67" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A67" s="40">
         <f>IF(B67="","",IF(D67=D65,A65+1,(D67*100)))</f>
         <v>207</v>
@@ -3107,7 +3107,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="68" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A68" s="40">
         <f t="shared" si="3"/>
         <v>208</v>
@@ -3134,7 +3134,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="69" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A69" s="40">
         <f t="shared" ref="A69" si="9">IF(B69="","",IF(D69=D68,A68+1,(D69*100)))</f>
         <v>209</v>
@@ -3161,7 +3161,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="70" spans="1:12" ht="19.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:12" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A70" s="40">
         <f>IF(B70="","",IF(D70=Sheet1!D68,Sheet1!A68+1,(D70*100)))</f>
         <v>209</v>
@@ -3190,7 +3190,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="71" spans="1:12" s="61" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:12" s="61" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A71" s="56">
         <f>IF(B71="","",IF(D71=D65,A65+1,(D71*100)))</f>
         <v>300</v>
@@ -3219,7 +3219,7 @@
       <c r="K71" s="58"/>
       <c r="L71" s="79"/>
     </row>
-    <row r="72" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A72" s="40">
         <f>IF(B72="","",IF(D72=D71,A71+1,(D72*100)))</f>
         <v>301</v>
@@ -3244,7 +3244,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="73" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A73" s="40">
         <f t="shared" ref="A73:A91" si="14">IF(B73="","",IF(D73=D72,A72+1,(D73*100)))</f>
         <v>302</v>
@@ -3269,7 +3269,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="74" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A74" s="40">
         <f t="shared" si="14"/>
         <v>303</v>
@@ -3294,7 +3294,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="75" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A75" s="40">
         <f t="shared" si="14"/>
         <v>304</v>
@@ -3319,7 +3319,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="76" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A76" s="40">
         <f t="shared" si="14"/>
         <v>305</v>
@@ -3347,7 +3347,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="77" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A77" s="40">
         <f t="shared" si="14"/>
         <v>306</v>
@@ -3369,7 +3369,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A78" s="40">
         <f t="shared" si="14"/>
         <v>307</v>
@@ -3391,7 +3391,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A79" s="40">
         <f>IF(B79="","",IF(D79=D78,A78+1,(D79*100)))</f>
         <v>308</v>
@@ -3413,7 +3413,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A80" s="40">
         <f t="shared" si="14"/>
         <v>309</v>
@@ -3435,7 +3435,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A81" s="40">
         <f t="shared" si="14"/>
         <v>310</v>
@@ -3457,7 +3457,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="1:12" ht="19.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:12" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A82" s="40">
         <f t="shared" si="14"/>
         <v>311</v>
@@ -3474,15 +3474,18 @@
       <c r="E82" s="39">
         <v>45613</v>
       </c>
+      <c r="F82" s="11">
+        <v>45616</v>
+      </c>
       <c r="G82" s="6">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L82" s="72" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="83" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A83" s="40">
         <f t="shared" si="14"/>
         <v>312</v>
@@ -3505,7 +3508,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A84" s="40">
         <f t="shared" si="14"/>
         <v>313</v>
@@ -3524,12 +3527,15 @@
         <f t="shared" si="8"/>
         <v>45613</v>
       </c>
+      <c r="F84" s="11">
+        <v>45616</v>
+      </c>
       <c r="G84" s="6">
         <f t="shared" si="13"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="85" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="85" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A85" s="40">
         <f t="shared" si="14"/>
         <v>314</v>
@@ -3553,7 +3559,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A86" s="40">
         <f t="shared" si="14"/>
         <v>315</v>
@@ -3574,7 +3580,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A87" s="40">
         <f t="shared" si="14"/>
         <v>316</v>
@@ -3597,7 +3603,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A88" s="40">
         <f t="shared" si="14"/>
         <v>317</v>
@@ -3615,7 +3621,7 @@
         <v>45614</v>
       </c>
     </row>
-    <row r="89" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A89" s="40">
         <f t="shared" si="14"/>
         <v>318</v>
@@ -3637,7 +3643,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A90" s="40">
         <f t="shared" si="14"/>
         <v>319</v>
@@ -3652,16 +3658,18 @@
         <f>IF(B90="","",D87)</f>
         <v>3</v>
       </c>
-      <c r="E90" s="39" t="str">
-        <f>IF(B90="","",IF(D90=D87,E87,E87+14))</f>
-        <v>`</v>
+      <c r="E90" s="39">
+        <v>45616</v>
+      </c>
+      <c r="F90" s="11">
+        <v>45616</v>
       </c>
       <c r="G90" s="6">
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A91" s="40">
         <f t="shared" si="14"/>
         <v>320</v>
@@ -3677,15 +3685,17 @@
         <v>3</v>
       </c>
       <c r="E91" s="39">
-        <v>45614</v>
-      </c>
-      <c r="F91" s="39"/>
+        <v>45616</v>
+      </c>
+      <c r="F91" s="39">
+        <v>45616</v>
+      </c>
       <c r="G91" s="6">
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A92" s="56" t="str">
         <f t="shared" ref="A92" si="15">IF(B92="","",IF(D92=D90,A90+1,(D92*100)))</f>
         <v/>
@@ -3699,7 +3709,7 @@
         <v/>
       </c>
     </row>
-    <row r="93" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A93" s="40" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -3717,7 +3727,7 @@
         <v/>
       </c>
     </row>
-    <row r="94" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A94" s="40" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -3735,7 +3745,7 @@
         <v/>
       </c>
     </row>
-    <row r="95" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A95" s="40" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -3753,7 +3763,7 @@
         <v/>
       </c>
     </row>
-    <row r="96" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A96" s="40" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -3771,7 +3781,7 @@
         <v/>
       </c>
     </row>
-    <row r="97" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A97" s="40" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -3789,7 +3799,7 @@
         <v/>
       </c>
     </row>
-    <row r="98" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A98" s="40" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -3807,7 +3817,7 @@
         <v/>
       </c>
     </row>
-    <row r="99" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A99" s="40" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -3825,7 +3835,7 @@
         <v/>
       </c>
     </row>
-    <row r="100" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A100" s="40" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -3843,7 +3853,7 @@
         <v/>
       </c>
     </row>
-    <row r="101" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A101" s="40" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -3861,7 +3871,7 @@
         <v/>
       </c>
     </row>
-    <row r="102" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A102" s="40" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -3879,7 +3889,7 @@
         <v/>
       </c>
     </row>
-    <row r="103" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A103" s="40" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -3897,7 +3907,7 @@
         <v/>
       </c>
     </row>
-    <row r="104" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A104" s="40" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -3915,7 +3925,7 @@
         <v/>
       </c>
     </row>
-    <row r="105" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A105" s="40" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -3933,7 +3943,7 @@
         <v/>
       </c>
     </row>
-    <row r="106" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A106" s="40" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -3951,7 +3961,7 @@
         <v/>
       </c>
     </row>
-    <row r="107" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A107" s="40" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -3969,7 +3979,7 @@
         <v/>
       </c>
     </row>
-    <row r="108" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A108" s="40" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -3987,7 +3997,7 @@
         <v/>
       </c>
     </row>
-    <row r="109" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A109" s="40" t="str">
         <f t="shared" ref="A109:A166" si="16">IF(B109="","",IF(D109=D108,A108+1,(D109*100)))</f>
         <v/>
@@ -4005,7 +4015,7 @@
         <v/>
       </c>
     </row>
-    <row r="110" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A110" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4023,7 +4033,7 @@
         <v/>
       </c>
     </row>
-    <row r="111" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A111" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4041,7 +4051,7 @@
         <v/>
       </c>
     </row>
-    <row r="112" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A112" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4059,7 +4069,7 @@
         <v/>
       </c>
     </row>
-    <row r="113" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A113" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4077,7 +4087,7 @@
         <v/>
       </c>
     </row>
-    <row r="114" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A114" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4095,7 +4105,7 @@
         <v/>
       </c>
     </row>
-    <row r="115" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A115" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4113,7 +4123,7 @@
         <v/>
       </c>
     </row>
-    <row r="116" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A116" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4131,7 +4141,7 @@
         <v/>
       </c>
     </row>
-    <row r="117" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A117" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4149,7 +4159,7 @@
         <v/>
       </c>
     </row>
-    <row r="118" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A118" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4167,7 +4177,7 @@
         <v/>
       </c>
     </row>
-    <row r="119" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A119" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4185,7 +4195,7 @@
         <v/>
       </c>
     </row>
-    <row r="120" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A120" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4203,7 +4213,7 @@
         <v/>
       </c>
     </row>
-    <row r="121" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A121" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4221,7 +4231,7 @@
         <v/>
       </c>
     </row>
-    <row r="122" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A122" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4239,7 +4249,7 @@
         <v/>
       </c>
     </row>
-    <row r="123" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A123" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4257,7 +4267,7 @@
         <v/>
       </c>
     </row>
-    <row r="124" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A124" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4275,7 +4285,7 @@
         <v/>
       </c>
     </row>
-    <row r="125" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A125" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4293,7 +4303,7 @@
         <v/>
       </c>
     </row>
-    <row r="126" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A126" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4311,7 +4321,7 @@
         <v/>
       </c>
     </row>
-    <row r="127" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A127" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4329,7 +4339,7 @@
         <v/>
       </c>
     </row>
-    <row r="128" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A128" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4347,7 +4357,7 @@
         <v/>
       </c>
     </row>
-    <row r="129" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A129" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4365,7 +4375,7 @@
         <v/>
       </c>
     </row>
-    <row r="130" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A130" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4383,7 +4393,7 @@
         <v/>
       </c>
     </row>
-    <row r="131" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A131" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4401,7 +4411,7 @@
         <v/>
       </c>
     </row>
-    <row r="132" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A132" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4419,7 +4429,7 @@
         <v/>
       </c>
     </row>
-    <row r="133" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A133" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4437,7 +4447,7 @@
         <v/>
       </c>
     </row>
-    <row r="134" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A134" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4455,7 +4465,7 @@
         <v/>
       </c>
     </row>
-    <row r="135" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A135" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4473,7 +4483,7 @@
         <v/>
       </c>
     </row>
-    <row r="136" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A136" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4491,7 +4501,7 @@
         <v/>
       </c>
     </row>
-    <row r="137" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A137" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4509,7 +4519,7 @@
         <v/>
       </c>
     </row>
-    <row r="138" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A138" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4527,7 +4537,7 @@
         <v/>
       </c>
     </row>
-    <row r="139" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A139" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4545,7 +4555,7 @@
         <v/>
       </c>
     </row>
-    <row r="140" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A140" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4563,7 +4573,7 @@
         <v/>
       </c>
     </row>
-    <row r="141" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A141" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4581,7 +4591,7 @@
         <v/>
       </c>
     </row>
-    <row r="142" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A142" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4599,7 +4609,7 @@
         <v/>
       </c>
     </row>
-    <row r="143" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A143" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4617,7 +4627,7 @@
         <v/>
       </c>
     </row>
-    <row r="144" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A144" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4635,7 +4645,7 @@
         <v/>
       </c>
     </row>
-    <row r="145" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A145" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4653,7 +4663,7 @@
         <v/>
       </c>
     </row>
-    <row r="146" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A146" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4671,7 +4681,7 @@
         <v/>
       </c>
     </row>
-    <row r="147" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A147" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4689,7 +4699,7 @@
         <v/>
       </c>
     </row>
-    <row r="148" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A148" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4707,7 +4717,7 @@
         <v/>
       </c>
     </row>
-    <row r="149" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A149" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4725,7 +4735,7 @@
         <v/>
       </c>
     </row>
-    <row r="150" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A150" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4743,7 +4753,7 @@
         <v/>
       </c>
     </row>
-    <row r="151" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A151" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4761,7 +4771,7 @@
         <v/>
       </c>
     </row>
-    <row r="152" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A152" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4779,7 +4789,7 @@
         <v/>
       </c>
     </row>
-    <row r="153" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A153" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4797,7 +4807,7 @@
         <v/>
       </c>
     </row>
-    <row r="154" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A154" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4815,7 +4825,7 @@
         <v/>
       </c>
     </row>
-    <row r="155" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A155" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4833,7 +4843,7 @@
         <v/>
       </c>
     </row>
-    <row r="156" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A156" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4851,7 +4861,7 @@
         <v/>
       </c>
     </row>
-    <row r="157" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A157" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4869,7 +4879,7 @@
         <v/>
       </c>
     </row>
-    <row r="158" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A158" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4887,7 +4897,7 @@
         <v/>
       </c>
     </row>
-    <row r="159" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A159" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4905,7 +4915,7 @@
         <v/>
       </c>
     </row>
-    <row r="160" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A160" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4923,7 +4933,7 @@
         <v/>
       </c>
     </row>
-    <row r="161" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A161" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4941,7 +4951,7 @@
         <v/>
       </c>
     </row>
-    <row r="162" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A162" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4959,7 +4969,7 @@
         <v/>
       </c>
     </row>
-    <row r="163" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A163" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4977,7 +4987,7 @@
         <v/>
       </c>
     </row>
-    <row r="164" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A164" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4995,7 +5005,7 @@
         <v/>
       </c>
     </row>
-    <row r="165" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A165" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -5013,7 +5023,7 @@
         <v/>
       </c>
     </row>
-    <row r="166" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A166" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -5033,6 +5043,11 @@
     </row>
   </sheetData>
   <mergeCells count="21">
+    <mergeCell ref="L34:L38"/>
+    <mergeCell ref="E62:G62"/>
+    <mergeCell ref="E63:G63"/>
+    <mergeCell ref="E64:G64"/>
+    <mergeCell ref="E58:G58"/>
     <mergeCell ref="E65:G65"/>
     <mergeCell ref="H10:H11"/>
     <mergeCell ref="H9:K9"/>
@@ -5049,11 +5064,6 @@
     <mergeCell ref="C10:C11"/>
     <mergeCell ref="F10:F11"/>
     <mergeCell ref="L9:L11"/>
-    <mergeCell ref="L34:L38"/>
-    <mergeCell ref="E62:G62"/>
-    <mergeCell ref="E63:G63"/>
-    <mergeCell ref="E64:G64"/>
-    <mergeCell ref="E58:G58"/>
   </mergeCells>
   <conditionalFormatting sqref="G54">
     <cfRule type="colorScale" priority="8">
@@ -5091,8 +5101,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G70">
-    <cfRule type="colorScale" priority="7">
+  <conditionalFormatting sqref="G67:G69 G14:G53 G59 G55:G57 G71:G166">
+    <cfRule type="colorScale" priority="18">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -5103,8 +5113,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G67:G69 G14:G53 G59 G55:G57 G71:G166">
-    <cfRule type="colorScale" priority="18">
+  <conditionalFormatting sqref="G70">
+    <cfRule type="colorScale" priority="7">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>

</xml_diff>

<commit_message>
Temp fix for breakroom not having puzzle
-update requirements doc
-temporarily commented out locks in breakroom, do not have a working puzzle to put into it.
-removed some locks to prevent soft locking self into a room
</commit_message>
<xml_diff>
--- a/Documents/project requirements spreadsheet.xlsx
+++ b/Documents/project requirements spreadsheet.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11110"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/soapmac/Documents/GitHub/Shattered-Protocols-Text-RPG/Shattered Protocols/Shattered-Protocols-Text-RPG/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Files\Documents\__ School\CS 3300- Software Development\Project (Group 1)\Shattered-Protocols-Text-RPG\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE46A757-6460-CC4F-9E9E-282D8A9E1569}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A232FA09-123C-43C6-B9F8-56AAAE26986F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15800" xr2:uid="{CAB5D44A-E176-404C-B398-BEAD2D9E6884}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" xr2:uid="{CAB5D44A-E176-404C-B398-BEAD2D9E6884}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="276" uniqueCount="141">
   <si>
     <t>Intro to Software Engineering</t>
   </si>
@@ -400,9 +400,6 @@
     <t>*If time, make room puzzles show when attempting to use a locked door or something</t>
   </si>
   <si>
-    <t>`</t>
-  </si>
-  <si>
     <t>Add additional Comments to Core Programming parts</t>
   </si>
   <si>
@@ -439,15 +436,9 @@
     <t>Test making Executable (How hard is it?)</t>
   </si>
   <si>
-    <t>*if time: Computer console setup for accessing puzzles rather than automatic</t>
-  </si>
-  <si>
     <t>Make Puzzle Nullable without breaking game (Room line 88)</t>
   </si>
   <si>
-    <t xml:space="preserve">Breakroom: If R2 door is unlocked use R4 puzzle, and the opposite. </t>
-  </si>
-  <si>
     <t>Seth and Juhan decided at the last minute that we just wont do automated testing.</t>
   </si>
   <si>
@@ -460,7 +451,22 @@
     <t>This was already happening last iteration, dont know why i thought it wasnt.</t>
   </si>
   <si>
-    <t>*if time have the game SHOW that doors are locked on entry</t>
+    <t>Tie Save system (gamestate.cs) into keyword system</t>
+  </si>
+  <si>
+    <t>*Completely forgot to do this</t>
+  </si>
+  <si>
+    <t>Remove Debug Outputs on Puzzles</t>
+  </si>
+  <si>
+    <t>Breakroom Puzzle</t>
+  </si>
+  <si>
+    <t>*Puzzle submitted, doesnt work and not added to room</t>
+  </si>
+  <si>
+    <t>If Breakroom puzzle is working, add it and uncomment door locks, otherwise remove door lock code</t>
   </si>
 </sst>
 </file>
@@ -737,7 +743,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="12" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="94">
+  <cellXfs count="95">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -979,6 +985,12 @@
     <xf numFmtId="16" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
     <xf numFmtId="14" fontId="13" fillId="7" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1012,11 +1024,8 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1360,121 +1369,121 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B900A37F-814E-4AF4-9047-E946E2A67EEB}">
-  <dimension ref="A1:L166"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:L162"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="15" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15.5" style="6" customWidth="1"/>
+    <col min="1" max="1" width="15.44140625" style="6" customWidth="1"/>
     <col min="2" max="2" width="61.33203125" style="5" customWidth="1"/>
-    <col min="3" max="3" width="17.1640625" style="6" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.109375" style="6" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12.6640625" style="6" customWidth="1"/>
-    <col min="5" max="5" width="15.83203125" style="6" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.77734375" style="6" bestFit="1" customWidth="1"/>
     <col min="6" max="7" width="12.6640625" style="6" customWidth="1"/>
-    <col min="8" max="8" width="16.1640625" style="6" customWidth="1"/>
+    <col min="8" max="8" width="16.109375" style="6" customWidth="1"/>
     <col min="9" max="11" width="12.6640625" style="6" customWidth="1"/>
-    <col min="12" max="12" width="173.83203125" style="72" customWidth="1"/>
-    <col min="13" max="16384" width="9.1640625" style="12"/>
+    <col min="12" max="12" width="173.77734375" style="72" customWidth="1"/>
+    <col min="13" max="16384" width="9.109375" style="12"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" s="26" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="84" t="s">
+    <row r="1" spans="1:12" s="26" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="86" t="s">
         <v>85</v>
       </c>
-      <c r="B1" s="85"/>
+      <c r="B1" s="87"/>
       <c r="C1" s="24"/>
-      <c r="D1" s="90" t="s">
+      <c r="D1" s="92" t="s">
         <v>86</v>
       </c>
-      <c r="E1" s="90"/>
-      <c r="F1" s="90"/>
-      <c r="G1" s="90"/>
-      <c r="H1" s="90"/>
-      <c r="I1" s="90"/>
-      <c r="J1" s="90"/>
-      <c r="K1" s="90"/>
+      <c r="E1" s="92"/>
+      <c r="F1" s="92"/>
+      <c r="G1" s="92"/>
+      <c r="H1" s="92"/>
+      <c r="I1" s="92"/>
+      <c r="J1" s="92"/>
+      <c r="K1" s="92"/>
       <c r="L1" s="64"/>
     </row>
-    <row r="2" spans="1:12" s="26" customFormat="1" ht="19" x14ac:dyDescent="0.2">
-      <c r="A2" s="86" t="s">
+    <row r="2" spans="1:12" s="26" customFormat="1" ht="18" x14ac:dyDescent="0.3">
+      <c r="A2" s="88" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="87"/>
+      <c r="B2" s="89"/>
       <c r="C2" s="24"/>
-      <c r="D2" s="90"/>
-      <c r="E2" s="90"/>
-      <c r="F2" s="90"/>
-      <c r="G2" s="90"/>
-      <c r="H2" s="90"/>
-      <c r="I2" s="90"/>
-      <c r="J2" s="90"/>
-      <c r="K2" s="90"/>
+      <c r="D2" s="92"/>
+      <c r="E2" s="92"/>
+      <c r="F2" s="92"/>
+      <c r="G2" s="92"/>
+      <c r="H2" s="92"/>
+      <c r="I2" s="92"/>
+      <c r="J2" s="92"/>
+      <c r="K2" s="92"/>
       <c r="L2" s="65"/>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3" s="41"/>
       <c r="B3" s="29"/>
       <c r="C3" s="12"/>
-      <c r="D3" s="90"/>
-      <c r="E3" s="90"/>
-      <c r="F3" s="90"/>
-      <c r="G3" s="90"/>
-      <c r="H3" s="90"/>
-      <c r="I3" s="90"/>
-      <c r="J3" s="90"/>
-      <c r="K3" s="90"/>
+      <c r="D3" s="92"/>
+      <c r="E3" s="92"/>
+      <c r="F3" s="92"/>
+      <c r="G3" s="92"/>
+      <c r="H3" s="92"/>
+      <c r="I3" s="92"/>
+      <c r="J3" s="92"/>
+      <c r="K3" s="92"/>
       <c r="L3" s="66"/>
     </row>
-    <row r="4" spans="1:12" s="7" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:12" s="7" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A4" s="42" t="s">
         <v>17</v>
       </c>
       <c r="B4" s="30" t="s">
         <v>39</v>
       </c>
-      <c r="D4" s="90"/>
-      <c r="E4" s="90"/>
-      <c r="F4" s="90"/>
-      <c r="G4" s="90"/>
-      <c r="H4" s="90"/>
-      <c r="I4" s="90"/>
-      <c r="J4" s="90"/>
-      <c r="K4" s="90"/>
+      <c r="D4" s="92"/>
+      <c r="E4" s="92"/>
+      <c r="F4" s="92"/>
+      <c r="G4" s="92"/>
+      <c r="H4" s="92"/>
+      <c r="I4" s="92"/>
+      <c r="J4" s="92"/>
+      <c r="K4" s="92"/>
       <c r="L4" s="67"/>
     </row>
-    <row r="5" spans="1:12" s="7" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:12" s="7" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A5" s="42" t="s">
         <v>18</v>
       </c>
       <c r="B5" s="30" t="s">
         <v>40</v>
       </c>
-      <c r="D5" s="90"/>
-      <c r="E5" s="90"/>
-      <c r="F5" s="90"/>
-      <c r="G5" s="90"/>
-      <c r="H5" s="90"/>
-      <c r="I5" s="90"/>
-      <c r="J5" s="90"/>
-      <c r="K5" s="90"/>
+      <c r="D5" s="92"/>
+      <c r="E5" s="92"/>
+      <c r="F5" s="92"/>
+      <c r="G5" s="92"/>
+      <c r="H5" s="92"/>
+      <c r="I5" s="92"/>
+      <c r="J5" s="92"/>
+      <c r="K5" s="92"/>
       <c r="L5" s="67"/>
     </row>
-    <row r="6" spans="1:12" s="7" customFormat="1" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:12" s="7" customFormat="1" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="43" t="s">
         <v>19</v>
       </c>
       <c r="B6" s="31" t="s">
         <v>84</v>
       </c>
-      <c r="D6" s="90"/>
-      <c r="E6" s="90"/>
-      <c r="F6" s="90"/>
-      <c r="G6" s="90"/>
-      <c r="H6" s="90"/>
-      <c r="I6" s="90"/>
-      <c r="J6" s="90"/>
-      <c r="K6" s="90"/>
+      <c r="D6" s="92"/>
+      <c r="E6" s="92"/>
+      <c r="F6" s="92"/>
+      <c r="G6" s="92"/>
+      <c r="H6" s="92"/>
+      <c r="I6" s="92"/>
+      <c r="J6" s="92"/>
+      <c r="K6" s="92"/>
       <c r="L6" s="68"/>
     </row>
-    <row r="7" spans="1:12" s="7" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:12" s="7" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A7" s="44"/>
       <c r="B7" s="2"/>
       <c r="C7" s="1"/>
@@ -1488,94 +1497,94 @@
       <c r="K7" s="1"/>
       <c r="L7" s="68"/>
     </row>
-    <row r="8" spans="1:12" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="83" t="s">
+    <row r="8" spans="1:12" s="7" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A8" s="85" t="s">
         <v>16</v>
       </c>
-      <c r="B8" s="83"/>
-      <c r="C8" s="83"/>
-      <c r="D8" s="83"/>
-      <c r="E8" s="83"/>
-      <c r="F8" s="83"/>
-      <c r="G8" s="83"/>
-      <c r="H8" s="83"/>
-      <c r="I8" s="83"/>
-      <c r="J8" s="83"/>
-      <c r="K8" s="83"/>
-      <c r="L8" s="83"/>
-    </row>
-    <row r="9" spans="1:12" s="7" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="B8" s="85"/>
+      <c r="C8" s="85"/>
+      <c r="D8" s="85"/>
+      <c r="E8" s="85"/>
+      <c r="F8" s="85"/>
+      <c r="G8" s="85"/>
+      <c r="H8" s="85"/>
+      <c r="I8" s="85"/>
+      <c r="J8" s="85"/>
+      <c r="K8" s="85"/>
+      <c r="L8" s="85"/>
+    </row>
+    <row r="9" spans="1:12" s="7" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
       <c r="B9" s="2"/>
-      <c r="C9" s="83" t="s">
+      <c r="C9" s="85" t="s">
         <v>15</v>
       </c>
-      <c r="D9" s="83"/>
-      <c r="E9" s="83"/>
-      <c r="F9" s="83"/>
+      <c r="D9" s="85"/>
+      <c r="E9" s="85"/>
+      <c r="F9" s="85"/>
       <c r="G9" s="1"/>
-      <c r="H9" s="83" t="s">
+      <c r="H9" s="85" t="s">
         <v>7</v>
       </c>
-      <c r="I9" s="83"/>
-      <c r="J9" s="83"/>
-      <c r="K9" s="83"/>
-      <c r="L9" s="91" t="s">
+      <c r="I9" s="85"/>
+      <c r="J9" s="85"/>
+      <c r="K9" s="85"/>
+      <c r="L9" s="93" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:12" s="7" customFormat="1" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:12" s="7" customFormat="1" ht="15.45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1"/>
       <c r="B10" s="2"/>
-      <c r="C10" s="82" t="s">
+      <c r="C10" s="84" t="s">
         <v>20</v>
       </c>
       <c r="D10" s="1"/>
-      <c r="E10" s="82" t="s">
+      <c r="E10" s="84" t="s">
         <v>55</v>
       </c>
-      <c r="F10" s="82" t="s">
+      <c r="F10" s="84" t="s">
         <v>56</v>
       </c>
-      <c r="G10" s="82" t="s">
+      <c r="G10" s="84" t="s">
         <v>57</v>
       </c>
-      <c r="H10" s="82" t="s">
+      <c r="H10" s="84" t="s">
         <v>4</v>
       </c>
-      <c r="I10" s="82" t="s">
+      <c r="I10" s="84" t="s">
         <v>20</v>
       </c>
-      <c r="J10" s="82" t="s">
+      <c r="J10" s="84" t="s">
         <v>5</v>
       </c>
       <c r="K10" s="1"/>
-      <c r="L10" s="91"/>
-    </row>
-    <row r="11" spans="1:12" s="7" customFormat="1" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="L10" s="93"/>
+    </row>
+    <row r="11" spans="1:12" s="7" customFormat="1" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>1</v>
       </c>
       <c r="B11" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="C11" s="82"/>
+      <c r="C11" s="84"/>
       <c r="D11" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E11" s="82"/>
-      <c r="F11" s="82"/>
-      <c r="G11" s="82"/>
-      <c r="H11" s="82"/>
-      <c r="I11" s="82"/>
-      <c r="J11" s="82"/>
+      <c r="E11" s="84"/>
+      <c r="F11" s="84"/>
+      <c r="G11" s="84"/>
+      <c r="H11" s="84"/>
+      <c r="I11" s="84"/>
+      <c r="J11" s="84"/>
       <c r="K11" s="25" t="s">
         <v>6</v>
       </c>
-      <c r="L11" s="91"/>
-    </row>
-    <row r="12" spans="1:12" s="55" customFormat="1" ht="52" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="88" t="s">
+      <c r="L11" s="93"/>
+    </row>
+    <row r="12" spans="1:12" s="55" customFormat="1" ht="45.6" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="90" t="s">
         <v>38</v>
       </c>
       <c r="B12" s="52"/>
@@ -1600,8 +1609,8 @@
       </c>
       <c r="L12" s="69"/>
     </row>
-    <row r="13" spans="1:12" s="3" customFormat="1" ht="61.5" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="89"/>
+    <row r="13" spans="1:12" s="3" customFormat="1" ht="61.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="91"/>
       <c r="B13" s="8"/>
       <c r="C13" s="10"/>
       <c r="D13" s="10" t="s">
@@ -1620,7 +1629,7 @@
       <c r="K13" s="10"/>
       <c r="L13" s="70"/>
     </row>
-    <row r="14" spans="1:12" s="21" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:12" s="21" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A14" s="45">
         <v>0</v>
       </c>
@@ -1651,13 +1660,13 @@
       <c r="K14" s="19"/>
       <c r="L14" s="71"/>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A15" s="46">
         <f>A14+1</f>
         <v>1</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C15" s="6" t="s">
         <v>35</v>
@@ -1676,7 +1685,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A16" s="46">
         <f t="shared" ref="A16:A32" si="0">A15+1</f>
         <v>2</v>
@@ -1701,7 +1710,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="17" spans="1:12" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:12" ht="15.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A17" s="46">
         <f t="shared" si="0"/>
         <v>3</v>
@@ -1726,7 +1735,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A18" s="46">
         <f t="shared" si="0"/>
         <v>4</v>
@@ -1751,7 +1760,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A19" s="46">
         <f t="shared" si="0"/>
         <v>5</v>
@@ -1776,7 +1785,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A20" s="46">
         <f t="shared" si="0"/>
         <v>6</v>
@@ -1801,7 +1810,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A21" s="46">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -1826,7 +1835,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A22" s="46">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -1851,13 +1860,13 @@
         <v>44</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A23" s="46">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C23" s="6" t="s">
         <v>42</v>
@@ -1876,13 +1885,13 @@
         <v>44</v>
       </c>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A24" s="46">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C24" s="23" t="s">
         <v>52</v>
@@ -1901,7 +1910,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A25" s="46">
         <f t="shared" si="0"/>
         <v>11</v>
@@ -1929,7 +1938,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A26" s="46">
         <f t="shared" si="0"/>
         <v>12</v>
@@ -1957,7 +1966,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A27" s="46">
         <f t="shared" si="0"/>
         <v>13</v>
@@ -1982,7 +1991,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A28" s="46">
         <f t="shared" si="0"/>
         <v>14</v>
@@ -2007,7 +2016,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A29" s="46">
         <f t="shared" si="0"/>
         <v>15</v>
@@ -2032,7 +2041,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A30" s="46">
         <f t="shared" si="0"/>
         <v>16</v>
@@ -2057,7 +2066,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="31" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="46">
         <f t="shared" si="0"/>
         <v>17</v>
@@ -2082,7 +2091,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="32" spans="1:12" s="14" customFormat="1" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:12" s="14" customFormat="1" ht="15.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A32" s="47">
         <f t="shared" si="0"/>
         <v>18</v>
@@ -2112,7 +2121,7 @@
       <c r="K32" s="10"/>
       <c r="L32" s="73"/>
     </row>
-    <row r="33" spans="1:12" s="17" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:12" s="17" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="48">
         <f>IF(D33=D32,A32+1,(D33*100))</f>
         <v>0</v>
@@ -2144,7 +2153,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A34" s="49">
         <f t="shared" ref="A34:A44" si="2">IF(D34=D33,A33+1,(D34*100))</f>
         <v>1</v>
@@ -2171,11 +2180,11 @@
       <c r="H34" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="L34" s="92" t="s">
+      <c r="L34" s="81" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A35" s="49">
         <f t="shared" si="2"/>
         <v>2</v>
@@ -2202,9 +2211,9 @@
       <c r="H35" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="L35" s="93"/>
-    </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="L35" s="82"/>
+    </row>
+    <row r="36" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A36" s="49">
         <f t="shared" si="2"/>
         <v>3</v>
@@ -2231,9 +2240,9 @@
       <c r="H36" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="L36" s="93"/>
-    </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="L36" s="82"/>
+    </row>
+    <row r="37" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A37" s="49">
         <f t="shared" si="2"/>
         <v>4</v>
@@ -2260,9 +2269,9 @@
       <c r="H37" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="L37" s="93"/>
-    </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="L37" s="82"/>
+    </row>
+    <row r="38" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A38" s="49">
         <f t="shared" si="2"/>
         <v>5</v>
@@ -2289,9 +2298,9 @@
       <c r="H38" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="L38" s="93"/>
-    </row>
-    <row r="39" spans="1:12" ht="32" x14ac:dyDescent="0.2">
+      <c r="L38" s="82"/>
+    </row>
+    <row r="39" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A39" s="49">
         <f t="shared" si="2"/>
         <v>6</v>
@@ -2322,7 +2331,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A40" s="49">
         <f t="shared" si="2"/>
         <v>7</v>
@@ -2353,7 +2362,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A41" s="49">
         <f t="shared" si="2"/>
         <v>8</v>
@@ -2384,7 +2393,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A42" s="49">
         <f t="shared" si="2"/>
         <v>9</v>
@@ -2415,7 +2424,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A43" s="49">
         <f t="shared" si="2"/>
         <v>10</v>
@@ -2446,7 +2455,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="44" spans="1:12" s="14" customFormat="1" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:12" s="14" customFormat="1" ht="15.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A44" s="50">
         <f t="shared" si="2"/>
         <v>11</v>
@@ -2480,7 +2489,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="45" spans="1:12" s="38" customFormat="1" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:12" s="38" customFormat="1" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A45" s="51">
         <f>IF(D45=D43,A43+1,(D45*100))</f>
         <v>100</v>
@@ -2509,7 +2518,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="46" spans="1:12" s="17" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:12" s="17" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="48">
         <f>IF(D46=D44,A44+1,(D46*100))</f>
         <v>100</v>
@@ -2537,9 +2546,9 @@
       <c r="K46" s="16"/>
       <c r="L46" s="78"/>
     </row>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A47" s="40">
-        <f t="shared" ref="A47:A108" si="3">IF(B47="","",IF(D47=D46,A46+1,(D47*100)))</f>
+        <f t="shared" ref="A47:A104" si="3">IF(B47="","",IF(D47=D46,A46+1,(D47*100)))</f>
         <v>101</v>
       </c>
       <c r="B47" s="5" t="s">
@@ -2558,14 +2567,14 @@
         <v>45600</v>
       </c>
       <c r="G47" s="6">
-        <f t="shared" ref="G47:G108" si="4">IF(B47="","",IF(AND(E47&gt;0,F47&gt;0),F47-E47,0))</f>
+        <f t="shared" ref="G47:G104" si="4">IF(B47="","",IF(AND(E47&gt;0,F47&gt;0),F47-E47,0))</f>
         <v>0</v>
       </c>
       <c r="H47" s="6" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A48" s="49">
         <f t="shared" si="3"/>
         <v>102</v>
@@ -2593,7 +2602,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="49" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A49" s="49">
         <f t="shared" si="3"/>
         <v>103</v>
@@ -2625,7 +2634,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="50" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A50" s="49">
         <f t="shared" si="3"/>
         <v>104</v>
@@ -2653,7 +2662,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="51" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A51" s="49">
         <f t="shared" si="3"/>
         <v>105</v>
@@ -2681,7 +2690,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="52" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A52" s="40">
         <f>IF(B52="","",IF(D52=D51,A51+1,(D52*100)))</f>
         <v>106</v>
@@ -2709,7 +2718,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="53" spans="1:12" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:12" ht="19.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="40" t="s">
         <v>100</v>
       </c>
@@ -2736,7 +2745,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="54" spans="1:12" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:12" ht="19.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" s="40">
         <f>IF(B54="","",IF(D54=Sheet1!D53,Sheet1!A53+1,(D54*100)))</f>
         <v>110.00000000000001</v>
@@ -2765,7 +2774,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="55" spans="1:12" s="61" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:12" s="61" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A55" s="56">
         <f>IF(B55="","",IF(D55=D52,A52+1,(D55*100)))</f>
         <v>200</v>
@@ -2794,7 +2803,7 @@
       <c r="K55" s="58"/>
       <c r="L55" s="79"/>
     </row>
-    <row r="56" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A56" s="40">
         <f>IF(B56="","",IF(D56=D53,A53+1,(D56*100)))</f>
         <v>200</v>
@@ -2822,7 +2831,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="57" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A57" s="40">
         <f>IF(B57="","",IF(D57=D62,A62+1,(D57*100)))</f>
         <v>202</v>
@@ -2851,7 +2860,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="58" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A58" s="40">
         <f t="shared" si="3"/>
         <v>203</v>
@@ -2863,22 +2872,22 @@
         <v>40</v>
       </c>
       <c r="D58" s="6">
-        <f t="shared" ref="D58:D120" si="5">IF(B58="","",D57)</f>
+        <f t="shared" ref="D58:D116" si="5">IF(B58="","",D57)</f>
         <v>2</v>
       </c>
-      <c r="E58" s="81" t="s">
+      <c r="E58" s="83" t="s">
         <v>112</v>
       </c>
-      <c r="F58" s="81"/>
-      <c r="G58" s="81"/>
+      <c r="F58" s="83"/>
+      <c r="G58" s="83"/>
       <c r="H58" s="6" t="s">
         <v>92</v>
       </c>
       <c r="L58" s="72" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="59" spans="1:12" x14ac:dyDescent="0.2">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="59" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A59" s="40">
         <f t="shared" si="3"/>
         <v>204</v>
@@ -2907,7 +2916,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="60" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A60" s="40">
         <f>IF(B60="","",IF(D60=D65,A65+1,(D60*100)))</f>
         <v>207</v>
@@ -2933,7 +2942,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="61" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A61" s="40">
         <f>IF(B61="","",IF(D61=D60,A60+1,(D61*100)))</f>
         <v>208</v>
@@ -2959,7 +2968,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="62" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A62" s="40">
         <f>IF(B62="","",IF(D62=D56,A56+1,(D62*100)))</f>
         <v>201</v>
@@ -2973,19 +2982,19 @@
       <c r="D62" s="6">
         <v>2</v>
       </c>
-      <c r="E62" s="81" t="s">
+      <c r="E62" s="83" t="s">
         <v>78</v>
       </c>
-      <c r="F62" s="81"/>
-      <c r="G62" s="81"/>
+      <c r="F62" s="83"/>
+      <c r="G62" s="83"/>
       <c r="H62" s="6" t="s">
         <v>92</v>
       </c>
       <c r="L62" s="72" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="63" spans="1:12" x14ac:dyDescent="0.2">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="63" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A63" s="40">
         <f>IF(B63="","",IF(D63=D61,A61+1,(D63*100)))</f>
         <v>209</v>
@@ -3000,16 +3009,16 @@
         <f>IF(B63="","",D61)</f>
         <v>2</v>
       </c>
-      <c r="E63" s="81" t="s">
+      <c r="E63" s="83" t="s">
         <v>78</v>
       </c>
-      <c r="F63" s="81"/>
-      <c r="G63" s="81"/>
+      <c r="F63" s="83"/>
+      <c r="G63" s="83"/>
       <c r="L63" s="72" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="64" spans="1:12" x14ac:dyDescent="0.2">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="64" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A64" s="40">
         <f>IF(B64="","",IF(D64=D59,A59+1,(D64*100)))</f>
         <v>205</v>
@@ -3024,13 +3033,13 @@
         <f>IF(B64="","",D59)</f>
         <v>2</v>
       </c>
-      <c r="E64" s="81" t="s">
+      <c r="E64" s="83" t="s">
         <v>78</v>
       </c>
-      <c r="F64" s="81"/>
-      <c r="G64" s="81"/>
-    </row>
-    <row r="65" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="F64" s="83"/>
+      <c r="G64" s="83"/>
+    </row>
+    <row r="65" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A65" s="40">
         <f>IF(B65="","",IF(D65=D64,A64+1,(D65*100)))</f>
         <v>206</v>
@@ -3045,16 +3054,16 @@
         <f>IF(B65="","",D64)</f>
         <v>2</v>
       </c>
-      <c r="E65" s="81" t="s">
+      <c r="E65" s="83" t="s">
         <v>112</v>
       </c>
-      <c r="F65" s="81"/>
-      <c r="G65" s="81"/>
+      <c r="F65" s="83"/>
+      <c r="G65" s="83"/>
       <c r="L65" s="72" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="66" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A66" s="40">
         <f>IF(B66="","",IF(D66=D63,A63+1,(D66*100)))</f>
         <v>210</v>
@@ -3080,7 +3089,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="67" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A67" s="40">
         <f>IF(B67="","",IF(D67=D65,A65+1,(D67*100)))</f>
         <v>207</v>
@@ -3107,7 +3116,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="68" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A68" s="40">
         <f t="shared" si="3"/>
         <v>208</v>
@@ -3123,7 +3132,7 @@
         <v>2</v>
       </c>
       <c r="E68" s="39">
-        <f t="shared" ref="E68:E116" si="8">IF(B68="","",IF(D68=D67,E67,E67+14))</f>
+        <f t="shared" ref="E68:E112" si="8">IF(B68="","",IF(D68=D67,E67,E67+14))</f>
         <v>45606</v>
       </c>
       <c r="F68" s="11">
@@ -3134,7 +3143,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="69" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A69" s="40">
         <f t="shared" ref="A69" si="9">IF(B69="","",IF(D69=D68,A68+1,(D69*100)))</f>
         <v>209</v>
@@ -3161,7 +3170,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="70" spans="1:12" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:12" ht="19.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A70" s="40">
         <f>IF(B70="","",IF(D70=Sheet1!D68,Sheet1!A68+1,(D70*100)))</f>
         <v>209</v>
@@ -3190,7 +3199,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="71" spans="1:12" s="61" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:12" s="61" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A71" s="56">
         <f>IF(B71="","",IF(D71=D65,A65+1,(D71*100)))</f>
         <v>300</v>
@@ -3210,7 +3219,7 @@
       </c>
       <c r="F71" s="58"/>
       <c r="G71" s="6">
-        <f t="shared" ref="G71:G91" si="13">IF(AND(E71&gt;0,F71&gt;0),F71-E71,0)</f>
+        <f t="shared" ref="G71:G87" si="13">IF(AND(E71&gt;0,F71&gt;0),F71-E71,0)</f>
         <v>0</v>
       </c>
       <c r="H71" s="58"/>
@@ -3219,13 +3228,13 @@
       <c r="K71" s="58"/>
       <c r="L71" s="79"/>
     </row>
-    <row r="72" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A72" s="40">
         <f>IF(B72="","",IF(D72=D71,A71+1,(D72*100)))</f>
         <v>301</v>
       </c>
       <c r="B72" s="5" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="C72" s="6" t="s">
         <v>40</v>
@@ -3244,9 +3253,9 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="73" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A73" s="40">
-        <f t="shared" ref="A73:A91" si="14">IF(B73="","",IF(D73=D72,A72+1,(D73*100)))</f>
+        <f t="shared" ref="A73:A90" si="14">IF(B73="","",IF(D73=D72,A72+1,(D73*100)))</f>
         <v>302</v>
       </c>
       <c r="B73" s="5" t="s">
@@ -3269,7 +3278,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="74" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A74" s="40">
         <f t="shared" si="14"/>
         <v>303</v>
@@ -3294,7 +3303,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="75" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A75" s="40">
         <f t="shared" si="14"/>
         <v>304</v>
@@ -3319,7 +3328,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="76" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A76" s="40">
         <f t="shared" si="14"/>
         <v>305</v>
@@ -3344,16 +3353,16 @@
         <v>-7</v>
       </c>
       <c r="L76" s="72" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="77" spans="1:12" x14ac:dyDescent="0.2">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="77" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A77" s="40">
         <f t="shared" si="14"/>
         <v>306</v>
       </c>
       <c r="B77" s="5" t="s">
-        <v>138</v>
+        <v>118</v>
       </c>
       <c r="C77" s="6" t="s">
         <v>40</v>
@@ -3362,6 +3371,9 @@
         <v>3</v>
       </c>
       <c r="E77" s="39">
+        <v>45613</v>
+      </c>
+      <c r="F77" s="11">
         <v>45613</v>
       </c>
       <c r="G77" s="6">
@@ -3369,16 +3381,16 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A78" s="40">
         <f t="shared" si="14"/>
         <v>307</v>
       </c>
       <c r="B78" s="5" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C78" s="6" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D78" s="6">
         <v>3</v>
@@ -3386,26 +3398,32 @@
       <c r="E78" s="39">
         <v>45613</v>
       </c>
+      <c r="F78" s="11">
+        <v>45616</v>
+      </c>
       <c r="G78" s="6">
         <f t="shared" si="13"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="79" spans="1:12" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="79" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A79" s="40">
-        <f>IF(B79="","",IF(D79=D78,A78+1,(D79*100)))</f>
+        <f t="shared" si="14"/>
         <v>308</v>
       </c>
       <c r="B79" s="5" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="C79" s="6" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D79" s="6">
         <v>3</v>
       </c>
       <c r="E79" s="39">
+        <v>45613</v>
+      </c>
+      <c r="F79" s="11">
         <v>45613</v>
       </c>
       <c r="G79" s="6">
@@ -3413,16 +3431,16 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:12" ht="19.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A80" s="40">
         <f t="shared" si="14"/>
         <v>309</v>
       </c>
       <c r="B80" s="5" t="s">
-        <v>122</v>
+        <v>37</v>
       </c>
       <c r="C80" s="6" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D80" s="6">
         <v>3</v>
@@ -3430,12 +3448,18 @@
       <c r="E80" s="39">
         <v>45613</v>
       </c>
+      <c r="F80" s="11">
+        <v>45616</v>
+      </c>
       <c r="G80" s="6">
         <f t="shared" si="13"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="81" spans="1:12" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+      <c r="L80" s="72" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="81" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A81" s="40">
         <f t="shared" si="14"/>
         <v>310</v>
@@ -3450,6 +3474,10 @@
         <v>3</v>
       </c>
       <c r="E81" s="39">
+        <f t="shared" si="8"/>
+        <v>45613</v>
+      </c>
+      <c r="F81" s="11">
         <v>45613</v>
       </c>
       <c r="G81" s="6">
@@ -3457,21 +3485,23 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="1:12" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A82" s="40">
         <f t="shared" si="14"/>
         <v>311</v>
       </c>
       <c r="B82" s="5" t="s">
-        <v>37</v>
+        <v>128</v>
       </c>
       <c r="C82" s="6" t="s">
         <v>43</v>
       </c>
       <c r="D82" s="6">
+        <f t="shared" si="5"/>
         <v>3</v>
       </c>
       <c r="E82" s="39">
+        <f t="shared" si="8"/>
         <v>45613</v>
       </c>
       <c r="F82" s="11">
@@ -3481,271 +3511,300 @@
         <f t="shared" si="13"/>
         <v>3</v>
       </c>
-      <c r="L82" s="72" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="83" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="83" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A83" s="40">
         <f t="shared" si="14"/>
         <v>312</v>
       </c>
       <c r="B83" s="5" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="C83" s="6" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D83" s="6">
+        <f t="shared" si="5"/>
         <v>3</v>
       </c>
-      <c r="E83" s="39">
-        <f t="shared" si="8"/>
-        <v>45613</v>
-      </c>
-      <c r="G83" s="6">
-        <f t="shared" si="13"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="84" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="E83" s="83" t="s">
+        <v>112</v>
+      </c>
+      <c r="F83" s="83"/>
+      <c r="G83" s="83"/>
+      <c r="L83" s="72" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="84" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A84" s="40">
         <f t="shared" si="14"/>
         <v>313</v>
       </c>
       <c r="B84" s="5" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="C84" s="6" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D84" s="6">
         <f t="shared" si="5"/>
         <v>3</v>
       </c>
       <c r="E84" s="39">
-        <f t="shared" si="8"/>
-        <v>45613</v>
+        <v>45615</v>
       </c>
       <c r="F84" s="11">
         <v>45616</v>
       </c>
       <c r="G84" s="6">
-        <f t="shared" si="13"/>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="85" spans="1:12" x14ac:dyDescent="0.2">
+        <f>IF(AND(E84&gt;0,F84&gt;0),F84-E84,0)</f>
+        <v>1</v>
+      </c>
+      <c r="L84" s="72" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="85" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A85" s="40">
         <f t="shared" si="14"/>
         <v>314</v>
       </c>
       <c r="B85" s="5" t="s">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="C85" s="6" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D85" s="6">
-        <f t="shared" si="5"/>
         <v>3</v>
       </c>
       <c r="E85" s="39">
-        <f t="shared" si="8"/>
-        <v>45613</v>
+        <v>45615</v>
+      </c>
+      <c r="F85" s="80">
+        <v>45616</v>
       </c>
       <c r="G85" s="6">
-        <f t="shared" si="13"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="86" spans="1:12" x14ac:dyDescent="0.2">
+        <f>IF(AND(E85&gt;0,F85&gt;0),F85-E85,0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="86" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A86" s="40">
         <f t="shared" si="14"/>
         <v>315</v>
       </c>
       <c r="B86" s="5" t="s">
-        <v>131</v>
+        <v>122</v>
+      </c>
+      <c r="C86" s="6" t="s">
+        <v>43</v>
       </c>
       <c r="D86" s="6">
         <f t="shared" si="5"/>
         <v>3</v>
       </c>
       <c r="E86" s="39">
-        <f t="shared" si="8"/>
-        <v>45613</v>
+        <v>45616</v>
+      </c>
+      <c r="F86" s="11">
+        <v>45616</v>
       </c>
       <c r="G86" s="6">
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A87" s="40">
         <f t="shared" si="14"/>
         <v>316</v>
       </c>
-      <c r="B87" s="5" t="s">
-        <v>133</v>
+      <c r="B87" s="5" t="str">
+        <f>"Iteration "&amp;D80&amp;" Test Report"</f>
+        <v>Iteration 3 Test Report</v>
       </c>
       <c r="C87" s="6" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D87" s="6">
-        <f t="shared" si="5"/>
         <v>3</v>
       </c>
-      <c r="E87" s="39" t="s">
-        <v>118</v>
+      <c r="E87" s="39">
+        <v>45616</v>
+      </c>
+      <c r="F87" s="39">
+        <v>45616</v>
       </c>
       <c r="G87" s="6">
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:12" s="61" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A88" s="40">
         <f t="shared" si="14"/>
         <v>317</v>
       </c>
-      <c r="B88" s="5" t="s">
-        <v>136</v>
-      </c>
-      <c r="C88" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="D88" s="6">
+      <c r="B88" s="57" t="str">
+        <f>"Iteration " &amp; D88 &amp; " Completion"</f>
+        <v>Iteration 3 Completion</v>
+      </c>
+      <c r="C88" s="58" t="s">
+        <v>35</v>
+      </c>
+      <c r="D88" s="58">
         <v>3</v>
       </c>
       <c r="E88" s="39">
-        <v>45614</v>
-      </c>
-    </row>
-    <row r="89" spans="1:12" x14ac:dyDescent="0.2">
+        <v>45616</v>
+      </c>
+      <c r="F88" s="58"/>
+      <c r="G88" s="6">
+        <f t="shared" ref="G88" si="15">IF(AND(E88&gt;0,F88&gt;0),F88-E88,0)</f>
+        <v>0</v>
+      </c>
+      <c r="H88" s="58"/>
+      <c r="I88" s="58"/>
+      <c r="J88" s="58"/>
+      <c r="K88" s="58"/>
+      <c r="L88" s="79"/>
+    </row>
+    <row r="89" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A89" s="40">
         <f t="shared" si="14"/>
         <v>318</v>
       </c>
       <c r="B89" s="5" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="C89" s="6" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D89" s="6">
         <v>3</v>
       </c>
       <c r="E89" s="39">
-        <v>45615</v>
+        <v>45616</v>
       </c>
       <c r="G89" s="6">
         <f>IF(AND(E89&gt;0,F89&gt;0),F89-E89,0)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A90" s="40">
         <f t="shared" si="14"/>
         <v>319</v>
       </c>
       <c r="B90" s="5" t="s">
-        <v>123</v>
+        <v>135</v>
       </c>
       <c r="C90" s="6" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="D90" s="6">
-        <f>IF(B90="","",D87)</f>
         <v>3</v>
       </c>
       <c r="E90" s="39">
         <v>45616</v>
       </c>
-      <c r="F90" s="11">
-        <v>45616</v>
-      </c>
       <c r="G90" s="6">
-        <f t="shared" si="13"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A91" s="40">
-        <f t="shared" si="14"/>
-        <v>320</v>
-      </c>
-      <c r="B91" s="5" t="str">
-        <f>"Iteration "&amp;D82&amp;" Test Report"</f>
-        <v>Iteration 3 Test Report</v>
-      </c>
-      <c r="C91" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="D91" s="6">
-        <v>3</v>
+    <row r="91" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A91" s="40" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="D91" s="6" t="str">
+        <f t="shared" si="5"/>
+        <v/>
       </c>
       <c r="E91" s="39">
         <v>45616</v>
       </c>
-      <c r="F91" s="39">
+      <c r="G91" s="6" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="92" spans="1:12" ht="30" x14ac:dyDescent="0.3">
+      <c r="A92" s="40" t="e">
+        <f t="shared" si="3"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="B92" s="94" t="s">
+        <v>140</v>
+      </c>
+      <c r="C92" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="D92" s="6" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+      <c r="E92" s="39">
+        <f t="shared" si="8"/>
         <v>45616</v>
       </c>
-      <c r="G91" s="6">
-        <f t="shared" si="13"/>
+      <c r="G92" s="6">
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A92" s="56" t="str">
-        <f t="shared" ref="A92" si="15">IF(B92="","",IF(D92=D90,A90+1,(D92*100)))</f>
-        <v/>
-      </c>
-      <c r="E92" s="39" t="str">
-        <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="G92" s="6" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-    </row>
-    <row r="93" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A93" s="40" t="str">
+    <row r="93" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A93" s="40" t="e">
         <f t="shared" si="3"/>
-        <v/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="B93" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="C93" s="6" t="s">
+        <v>42</v>
       </c>
       <c r="D93" s="6" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="E93" s="39" t="str">
+      <c r="E93" s="39">
         <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="G93" s="6" t="str">
+        <v>45616</v>
+      </c>
+      <c r="G93" s="6">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-    </row>
-    <row r="94" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A94" s="40" t="str">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="94" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A94" s="40" t="e">
         <f t="shared" si="3"/>
-        <v/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="B94" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="C94" s="6" t="s">
+        <v>42</v>
       </c>
       <c r="D94" s="6" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="E94" s="39" t="str">
+      <c r="E94" s="39">
         <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="G94" s="6" t="str">
+        <v>45616</v>
+      </c>
+      <c r="G94" s="6">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-    </row>
-    <row r="95" spans="1:12" x14ac:dyDescent="0.2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="95" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A95" s="40" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -3763,7 +3822,7 @@
         <v/>
       </c>
     </row>
-    <row r="96" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A96" s="40" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -3781,7 +3840,7 @@
         <v/>
       </c>
     </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A97" s="40" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -3799,7 +3858,7 @@
         <v/>
       </c>
     </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A98" s="40" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -3817,7 +3876,7 @@
         <v/>
       </c>
     </row>
-    <row r="99" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A99" s="40" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -3835,7 +3894,7 @@
         <v/>
       </c>
     </row>
-    <row r="100" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A100" s="40" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -3853,7 +3912,7 @@
         <v/>
       </c>
     </row>
-    <row r="101" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A101" s="40" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -3871,7 +3930,7 @@
         <v/>
       </c>
     </row>
-    <row r="102" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A102" s="40" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -3889,7 +3948,7 @@
         <v/>
       </c>
     </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A103" s="40" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -3907,7 +3966,7 @@
         <v/>
       </c>
     </row>
-    <row r="104" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A104" s="40" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -3925,9 +3984,9 @@
         <v/>
       </c>
     </row>
-    <row r="105" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A105" s="40" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" ref="A105:A162" si="16">IF(B105="","",IF(D105=D104,A104+1,(D105*100)))</f>
         <v/>
       </c>
       <c r="D105" s="6" t="str">
@@ -3939,13 +3998,13 @@
         <v/>
       </c>
       <c r="G105" s="6" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-    </row>
-    <row r="106" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" ref="G105:G162" si="17">IF(B105="","",IF(AND(E105&gt;0,F105&gt;0),F105-E105,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="106" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A106" s="40" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="D106" s="6" t="str">
@@ -3957,13 +4016,13 @@
         <v/>
       </c>
       <c r="G106" s="6" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-    </row>
-    <row r="107" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="17"/>
+        <v/>
+      </c>
+    </row>
+    <row r="107" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A107" s="40" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="D107" s="6" t="str">
@@ -3975,13 +4034,13 @@
         <v/>
       </c>
       <c r="G107" s="6" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-    </row>
-    <row r="108" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="17"/>
+        <v/>
+      </c>
+    </row>
+    <row r="108" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A108" s="40" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="D108" s="6" t="str">
@@ -3993,13 +4052,13 @@
         <v/>
       </c>
       <c r="G108" s="6" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-    </row>
-    <row r="109" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="17"/>
+        <v/>
+      </c>
+    </row>
+    <row r="109" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A109" s="40" t="str">
-        <f t="shared" ref="A109:A166" si="16">IF(B109="","",IF(D109=D108,A108+1,(D109*100)))</f>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="D109" s="6" t="str">
@@ -4011,11 +4070,11 @@
         <v/>
       </c>
       <c r="G109" s="6" t="str">
-        <f t="shared" ref="G109:G166" si="17">IF(B109="","",IF(AND(E109&gt;0,F109&gt;0),F109-E109,0))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="110" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="17"/>
+        <v/>
+      </c>
+    </row>
+    <row r="110" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A110" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4033,7 +4092,7 @@
         <v/>
       </c>
     </row>
-    <row r="111" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A111" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4051,7 +4110,7 @@
         <v/>
       </c>
     </row>
-    <row r="112" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A112" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4069,7 +4128,7 @@
         <v/>
       </c>
     </row>
-    <row r="113" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A113" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4079,7 +4138,7 @@
         <v/>
       </c>
       <c r="E113" s="39" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" ref="E113:E162" si="18">IF(B113="","",IF(D113=D112,E112,E112+14))</f>
         <v/>
       </c>
       <c r="G113" s="6" t="str">
@@ -4087,7 +4146,7 @@
         <v/>
       </c>
     </row>
-    <row r="114" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A114" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4097,7 +4156,7 @@
         <v/>
       </c>
       <c r="E114" s="39" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="G114" s="6" t="str">
@@ -4105,7 +4164,7 @@
         <v/>
       </c>
     </row>
-    <row r="115" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A115" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4115,7 +4174,7 @@
         <v/>
       </c>
       <c r="E115" s="39" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="G115" s="6" t="str">
@@ -4123,7 +4182,7 @@
         <v/>
       </c>
     </row>
-    <row r="116" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A116" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4133,7 +4192,7 @@
         <v/>
       </c>
       <c r="E116" s="39" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="G116" s="6" t="str">
@@ -4141,17 +4200,17 @@
         <v/>
       </c>
     </row>
-    <row r="117" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A117" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="D117" s="6" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" ref="D117:D162" si="19">IF(B117="","",D116)</f>
         <v/>
       </c>
       <c r="E117" s="39" t="str">
-        <f t="shared" ref="E117:E166" si="18">IF(B117="","",IF(D117=D116,E116,E116+14))</f>
+        <f t="shared" si="18"/>
         <v/>
       </c>
       <c r="G117" s="6" t="str">
@@ -4159,13 +4218,13 @@
         <v/>
       </c>
     </row>
-    <row r="118" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A118" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="D118" s="6" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="E118" s="39" t="str">
@@ -4177,13 +4236,13 @@
         <v/>
       </c>
     </row>
-    <row r="119" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A119" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="D119" s="6" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="E119" s="39" t="str">
@@ -4195,13 +4254,13 @@
         <v/>
       </c>
     </row>
-    <row r="120" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A120" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="D120" s="6" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="E120" s="39" t="str">
@@ -4213,13 +4272,13 @@
         <v/>
       </c>
     </row>
-    <row r="121" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A121" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="D121" s="6" t="str">
-        <f t="shared" ref="D121:D166" si="19">IF(B121="","",D120)</f>
+        <f t="shared" si="19"/>
         <v/>
       </c>
       <c r="E121" s="39" t="str">
@@ -4231,7 +4290,7 @@
         <v/>
       </c>
     </row>
-    <row r="122" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A122" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4249,7 +4308,7 @@
         <v/>
       </c>
     </row>
-    <row r="123" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A123" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4267,7 +4326,7 @@
         <v/>
       </c>
     </row>
-    <row r="124" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A124" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4285,7 +4344,7 @@
         <v/>
       </c>
     </row>
-    <row r="125" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A125" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4303,7 +4362,7 @@
         <v/>
       </c>
     </row>
-    <row r="126" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A126" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4321,7 +4380,7 @@
         <v/>
       </c>
     </row>
-    <row r="127" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A127" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4339,7 +4398,7 @@
         <v/>
       </c>
     </row>
-    <row r="128" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A128" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4357,7 +4416,7 @@
         <v/>
       </c>
     </row>
-    <row r="129" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A129" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4375,7 +4434,7 @@
         <v/>
       </c>
     </row>
-    <row r="130" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A130" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4393,7 +4452,7 @@
         <v/>
       </c>
     </row>
-    <row r="131" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A131" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4411,7 +4470,7 @@
         <v/>
       </c>
     </row>
-    <row r="132" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A132" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4429,7 +4488,7 @@
         <v/>
       </c>
     </row>
-    <row r="133" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A133" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4447,7 +4506,7 @@
         <v/>
       </c>
     </row>
-    <row r="134" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A134" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4465,7 +4524,7 @@
         <v/>
       </c>
     </row>
-    <row r="135" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A135" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4483,7 +4542,7 @@
         <v/>
       </c>
     </row>
-    <row r="136" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A136" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4501,7 +4560,7 @@
         <v/>
       </c>
     </row>
-    <row r="137" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A137" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4519,7 +4578,7 @@
         <v/>
       </c>
     </row>
-    <row r="138" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A138" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4537,7 +4596,7 @@
         <v/>
       </c>
     </row>
-    <row r="139" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A139" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4555,7 +4614,7 @@
         <v/>
       </c>
     </row>
-    <row r="140" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A140" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4573,7 +4632,7 @@
         <v/>
       </c>
     </row>
-    <row r="141" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A141" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4591,7 +4650,7 @@
         <v/>
       </c>
     </row>
-    <row r="142" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A142" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4609,7 +4668,7 @@
         <v/>
       </c>
     </row>
-    <row r="143" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="143" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A143" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4627,7 +4686,7 @@
         <v/>
       </c>
     </row>
-    <row r="144" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="144" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A144" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4645,7 +4704,7 @@
         <v/>
       </c>
     </row>
-    <row r="145" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A145" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4663,7 +4722,7 @@
         <v/>
       </c>
     </row>
-    <row r="146" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A146" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4681,7 +4740,7 @@
         <v/>
       </c>
     </row>
-    <row r="147" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="147" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A147" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4699,7 +4758,7 @@
         <v/>
       </c>
     </row>
-    <row r="148" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="148" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A148" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4717,7 +4776,7 @@
         <v/>
       </c>
     </row>
-    <row r="149" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="149" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A149" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4735,7 +4794,7 @@
         <v/>
       </c>
     </row>
-    <row r="150" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="150" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A150" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4753,7 +4812,7 @@
         <v/>
       </c>
     </row>
-    <row r="151" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="151" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A151" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4771,7 +4830,7 @@
         <v/>
       </c>
     </row>
-    <row r="152" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="152" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A152" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4789,7 +4848,7 @@
         <v/>
       </c>
     </row>
-    <row r="153" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="153" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A153" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4807,7 +4866,7 @@
         <v/>
       </c>
     </row>
-    <row r="154" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="154" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A154" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4825,7 +4884,7 @@
         <v/>
       </c>
     </row>
-    <row r="155" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="155" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A155" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4843,7 +4902,7 @@
         <v/>
       </c>
     </row>
-    <row r="156" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="156" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A156" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4861,7 +4920,7 @@
         <v/>
       </c>
     </row>
-    <row r="157" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="157" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A157" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4879,7 +4938,7 @@
         <v/>
       </c>
     </row>
-    <row r="158" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="158" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A158" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4897,7 +4956,7 @@
         <v/>
       </c>
     </row>
-    <row r="159" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="159" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A159" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4915,7 +4974,7 @@
         <v/>
       </c>
     </row>
-    <row r="160" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="160" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A160" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4933,7 +4992,7 @@
         <v/>
       </c>
     </row>
-    <row r="161" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="161" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A161" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4951,7 +5010,7 @@
         <v/>
       </c>
     </row>
-    <row r="162" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="162" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A162" s="40" t="str">
         <f t="shared" si="16"/>
         <v/>
@@ -4969,85 +5028,9 @@
         <v/>
       </c>
     </row>
-    <row r="163" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A163" s="40" t="str">
-        <f t="shared" si="16"/>
-        <v/>
-      </c>
-      <c r="D163" s="6" t="str">
-        <f t="shared" si="19"/>
-        <v/>
-      </c>
-      <c r="E163" s="39" t="str">
-        <f t="shared" si="18"/>
-        <v/>
-      </c>
-      <c r="G163" s="6" t="str">
-        <f t="shared" si="17"/>
-        <v/>
-      </c>
-    </row>
-    <row r="164" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A164" s="40" t="str">
-        <f t="shared" si="16"/>
-        <v/>
-      </c>
-      <c r="D164" s="6" t="str">
-        <f t="shared" si="19"/>
-        <v/>
-      </c>
-      <c r="E164" s="39" t="str">
-        <f t="shared" si="18"/>
-        <v/>
-      </c>
-      <c r="G164" s="6" t="str">
-        <f t="shared" si="17"/>
-        <v/>
-      </c>
-    </row>
-    <row r="165" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A165" s="40" t="str">
-        <f t="shared" si="16"/>
-        <v/>
-      </c>
-      <c r="D165" s="6" t="str">
-        <f t="shared" si="19"/>
-        <v/>
-      </c>
-      <c r="E165" s="39" t="str">
-        <f t="shared" si="18"/>
-        <v/>
-      </c>
-      <c r="G165" s="6" t="str">
-        <f t="shared" si="17"/>
-        <v/>
-      </c>
-    </row>
-    <row r="166" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A166" s="40" t="str">
-        <f t="shared" si="16"/>
-        <v/>
-      </c>
-      <c r="D166" s="6" t="str">
-        <f t="shared" si="19"/>
-        <v/>
-      </c>
-      <c r="E166" s="39" t="str">
-        <f t="shared" si="18"/>
-        <v/>
-      </c>
-      <c r="G166" s="6" t="str">
-        <f t="shared" si="17"/>
-        <v/>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="21">
-    <mergeCell ref="L34:L38"/>
-    <mergeCell ref="E62:G62"/>
-    <mergeCell ref="E63:G63"/>
-    <mergeCell ref="E64:G64"/>
-    <mergeCell ref="E58:G58"/>
+  <mergeCells count="22">
+    <mergeCell ref="E83:G83"/>
     <mergeCell ref="E65:G65"/>
     <mergeCell ref="H10:H11"/>
     <mergeCell ref="H9:K9"/>
@@ -5064,6 +5047,11 @@
     <mergeCell ref="C10:C11"/>
     <mergeCell ref="F10:F11"/>
     <mergeCell ref="L9:L11"/>
+    <mergeCell ref="L34:L38"/>
+    <mergeCell ref="E62:G62"/>
+    <mergeCell ref="E63:G63"/>
+    <mergeCell ref="E64:G64"/>
+    <mergeCell ref="E58:G58"/>
   </mergeCells>
   <conditionalFormatting sqref="G54">
     <cfRule type="colorScale" priority="8">
@@ -5089,20 +5077,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G66:G1048576 G59:G61 G10:G57">
+  <conditionalFormatting sqref="G66:G82 G59:G61 G10:G57 G84:G1048576">
     <cfRule type="colorScale" priority="4">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G67:G69 G14:G53 G59 G55:G57 G71:G166">
-    <cfRule type="colorScale" priority="18">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -5125,6 +5101,18 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="G67:G69 G14:G53 G59 G55:G57 G71:G82 G84:G162">
+    <cfRule type="colorScale" priority="30">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Updated Dates Requirements Sheet
</commit_message>
<xml_diff>
--- a/Documents/project requirements spreadsheet.xlsx
+++ b/Documents/project requirements spreadsheet.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11110"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Files\Documents\__ School\CS 3300- Software Development\Project (Group 1)\Shattered-Protocols-Text-RPG\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/soapmac/Documents/GitHub/Shattered-Protocols-Text-RPG/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5EEDE5B-F5D4-4A5A-814E-A2489C5B815F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{574E95E1-3044-4D41-9F68-482E3F2C9BD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="29016" windowHeight="15816" xr2:uid="{CAB5D44A-E176-404C-B398-BEAD2D9E6884}"/>
+    <workbookView xWindow="-38260" yWindow="-1400" windowWidth="38080" windowHeight="20780" xr2:uid="{CAB5D44A-E176-404C-B398-BEAD2D9E6884}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="125">
   <si>
     <t>Intro to Software Engineering</t>
   </si>
@@ -200,10 +200,6 @@
     <t>Initial Iteration due date moved from 10/15/24  to 10/31/24 to reorganize. Due to Iteration 0 team conflicts.</t>
   </si>
   <si>
-    <t>Communication, organizational and scheduling issues prevented earlier completion of the iteration.
-Many parts were completed fairly early, but team conflicts prevented Iteration from properly resolving.</t>
-  </si>
-  <si>
     <t>Project Idea Agreement</t>
   </si>
   <si>
@@ -219,17 +215,6 @@
     <t>Setup Puzzle Object Framework</t>
   </si>
   <si>
-    <t xml:space="preserve">Came up with 1 concept only, and very bare bones concept. Requirement should have been better defined. </t>
-  </si>
-  <si>
-    <t>Technically Added late to iteration as a better way of having rooms.
-Was part of a section of Git commits that I had not published due to team conflict issues (Uncertain if i was remaining with the team). So Actual completion date unknown</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Note: Original requirement and submission date were for the base objects setup, with intent to refine in future iterations. Submission of polished components was 10/18 technically 7 days past target due date.
-The objects were refined significantly during this time period, but not submitted to team Git due to team conflict and organizational concerns, and considering leaving the team. </t>
-  </si>
-  <si>
     <t>Come up with Puzzle concepts*</t>
   </si>
   <si>
@@ -368,25 +353,13 @@
     <t>Make Puzzle Nullable without breaking game (Room line 88)</t>
   </si>
   <si>
-    <t>Seth and Juhan decided at the last minute that we just wont do automated testing.</t>
-  </si>
-  <si>
-    <t>I ended up having to do a LOT of code this iteration, so pushing this off for future iteration</t>
-  </si>
-  <si>
     <t>Add new Puzzle for Breakroom</t>
   </si>
   <si>
-    <t>This was already happening last iteration, dont know why i thought it wasnt.</t>
-  </si>
-  <si>
-    <t>*Completely forgot to do this</t>
-  </si>
-  <si>
     <t>Remove Debug Outputs on Puzzles</t>
   </si>
   <si>
-    <t>*Puzzle submitted, doesnt work and not added to room</t>
+    <t>*if time Tie Save system (gamestate.cs) into keyword system</t>
   </si>
   <si>
     <t>Fix Binarysearch</t>
@@ -417,6 +390,28 @@
   </si>
   <si>
     <t>Final Submissions</t>
+  </si>
+  <si>
+    <t>Technically Added late to iteration as a better way of having rooms.</t>
+  </si>
+  <si>
+    <t>Taylor needed more time,  so pushing this off for future iteration</t>
+  </si>
+  <si>
+    <t>Seth decided not to continue with creating  automated testing as the project is too small. Great idea for the future!</t>
+  </si>
+  <si>
+    <t>Communication, organizational and scheduling issues prevented earlier completion of the iteration.</t>
+  </si>
+  <si>
+    <t>*Taylor  forgot to do this</t>
+  </si>
+  <si>
+    <t>*Puzzle submitted, doesnt work yet and not added to room</t>
+  </si>
+  <si>
+    <t>Note: Original requirement and submission date were for the base objects setup, with intent to refine in future iterations. Submission of polished components was 10/18 technically 7 days past target due date.
+The objects were refined significantly during this time period, but not submitted to team Git due to organizational concerns.</t>
   </si>
 </sst>
 </file>
@@ -427,7 +422,7 @@
     <numFmt numFmtId="164" formatCode="&quot;IT-&quot;0&quot;.&quot;00"/>
     <numFmt numFmtId="165" formatCode="&quot;Class&quot;00"/>
   </numFmts>
-  <fonts count="13" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -516,6 +511,12 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="7">
@@ -681,7 +682,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="11" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="88">
+  <cellXfs count="89">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -943,6 +944,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="14" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1286,22 +1290,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B900A37F-814E-4AF4-9047-E946E2A67EEB}">
-  <dimension ref="A1:H135"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="15" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:H143"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="15.44140625" style="6" customWidth="1"/>
+    <col min="1" max="1" width="15.5" style="6" customWidth="1"/>
     <col min="2" max="2" width="61.33203125" style="5" customWidth="1"/>
-    <col min="3" max="3" width="17.109375" style="6" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.1640625" style="6" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12.6640625" style="6" customWidth="1"/>
-    <col min="5" max="5" width="15.77734375" style="6" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.83203125" style="6" bestFit="1" customWidth="1"/>
     <col min="6" max="7" width="12.6640625" style="6" customWidth="1"/>
-    <col min="8" max="8" width="173.77734375" style="63" customWidth="1"/>
-    <col min="9" max="16384" width="9.109375" style="12"/>
+    <col min="8" max="8" width="173.83203125" style="63" customWidth="1"/>
+    <col min="9" max="16384" width="9.1640625" style="12"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="22" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" s="22" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="77" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="B1" s="78"/>
       <c r="C1" s="36" t="s">
@@ -1315,11 +1319,11 @@
         <v>12</v>
       </c>
       <c r="G1" s="26" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="H1" s="57"/>
     </row>
-    <row r="2" spans="1:8" s="22" customFormat="1" ht="18" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" s="22" customFormat="1" ht="19" x14ac:dyDescent="0.2">
       <c r="A2" s="79" t="s">
         <v>0</v>
       </c>
@@ -1333,7 +1337,7 @@
       <c r="G2" s="71"/>
       <c r="H2" s="58"/>
     </row>
-    <row r="3" spans="1:8" s="7" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" s="7" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A3" s="38"/>
       <c r="B3" s="2"/>
       <c r="C3" s="1"/>
@@ -1343,7 +1347,7 @@
       <c r="G3" s="1"/>
       <c r="H3" s="59"/>
     </row>
-    <row r="4" spans="1:8" s="7" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" s="7" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1"/>
       <c r="B4" s="2"/>
       <c r="C4" s="84" t="s">
@@ -1357,7 +1361,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:8" s="7" customFormat="1" ht="15.45" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" s="7" customFormat="1" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="1"/>
       <c r="B5" s="2"/>
       <c r="C5" s="83" t="s">
@@ -1375,7 +1379,7 @@
       </c>
       <c r="H5" s="74"/>
     </row>
-    <row r="6" spans="1:8" s="7" customFormat="1" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" s="7" customFormat="1" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>1</v>
       </c>
@@ -1391,7 +1395,7 @@
       <c r="G6" s="83"/>
       <c r="H6" s="74"/>
     </row>
-    <row r="7" spans="1:8" s="48" customFormat="1" ht="45.6" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" s="48" customFormat="1" ht="52" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A7" s="81" t="s">
         <v>31</v>
       </c>
@@ -1409,7 +1413,7 @@
       <c r="G7" s="19"/>
       <c r="H7" s="60"/>
     </row>
-    <row r="8" spans="1:8" s="3" customFormat="1" ht="61.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" s="3" customFormat="1" ht="61.5" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="82"/>
       <c r="B8" s="8"/>
       <c r="C8" s="10"/>
@@ -1423,12 +1427,12 @@
       <c r="G8" s="10"/>
       <c r="H8" s="61"/>
     </row>
-    <row r="9" spans="1:8" s="21" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" s="21" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A9" s="39">
         <v>0</v>
       </c>
       <c r="B9" s="18" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C9" s="19" t="s">
         <v>28</v>
@@ -1448,13 +1452,13 @@
       </c>
       <c r="H9" s="62"/>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A10" s="40">
         <f>A9+1</f>
         <v>1</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="C10" s="6" t="s">
         <v>28</v>
@@ -1473,7 +1477,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A11" s="40">
         <f t="shared" ref="A11:A27" si="0">A10+1</f>
         <v>2</v>
@@ -1490,15 +1494,16 @@
       <c r="E11" s="11">
         <v>45628</v>
       </c>
-      <c r="F11" s="11">
-        <v>45628</v>
+      <c r="F11" s="11" t="str">
+        <f>IF(F95&gt;0,F95,"")</f>
+        <v/>
       </c>
       <c r="G11" s="6">
         <f>IF(AND(E11&gt;0,ISNUMBER(F11)),F11-E11,0)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="15.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A12" s="40">
         <f t="shared" si="0"/>
         <v>3</v>
@@ -1507,7 +1512,7 @@
         <v>29</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="D12" s="6" t="s">
         <v>36</v>
@@ -1516,14 +1521,15 @@
         <v>45628</v>
       </c>
       <c r="F12" s="11">
+        <f t="shared" ref="F12:F19" si="1">IF(F96&gt;0,F96,"")</f>
         <v>45628</v>
       </c>
       <c r="G12" s="6">
-        <f t="shared" ref="G12:G21" si="1">IF(AND(E12&gt;0,ISNUMBER(F12)),F12-E12,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+        <f t="shared" ref="G12:G21" si="2">IF(AND(E12&gt;0,ISNUMBER(F12)),F12-E12,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" s="40">
         <f t="shared" si="0"/>
         <v>4</v>
@@ -1541,14 +1547,15 @@
         <v>45628</v>
       </c>
       <c r="F13" s="11">
+        <f t="shared" si="1"/>
         <v>45628</v>
       </c>
       <c r="G13" s="6">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14" s="40">
         <f t="shared" si="0"/>
         <v>5</v>
@@ -1566,14 +1573,15 @@
         <v>45628</v>
       </c>
       <c r="F14" s="11">
+        <f t="shared" si="1"/>
         <v>45628</v>
       </c>
       <c r="G14" s="6">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A15" s="40">
         <f t="shared" si="0"/>
         <v>6</v>
@@ -1591,14 +1599,15 @@
         <v>45628</v>
       </c>
       <c r="F15" s="11">
+        <f t="shared" si="1"/>
         <v>45628</v>
       </c>
       <c r="G15" s="6">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A16" s="40">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -1616,14 +1625,15 @@
         <v>45628</v>
       </c>
       <c r="F16" s="11">
+        <f t="shared" si="1"/>
         <v>45628</v>
       </c>
       <c r="G16" s="6">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A17" s="40">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -1641,21 +1651,21 @@
         <v>45628</v>
       </c>
       <c r="F17" s="11">
-        <f>IF(F94&gt;0,F94,"")</f>
+        <f t="shared" si="1"/>
         <v>45607</v>
       </c>
       <c r="G17" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>-21</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A18" s="40">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="C18" s="6" t="s">
         <v>34</v>
@@ -1667,20 +1677,21 @@
         <v>45628</v>
       </c>
       <c r="F18" s="11">
+        <f t="shared" si="1"/>
         <v>45628</v>
       </c>
       <c r="G18" s="6">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A19" s="40">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="C19" s="6" t="s">
         <v>33</v>
@@ -1691,21 +1702,22 @@
       <c r="E19" s="11">
         <v>45628</v>
       </c>
-      <c r="F19" s="11">
-        <v>45628</v>
+      <c r="F19" s="11" t="str">
+        <f t="shared" si="1"/>
+        <v/>
       </c>
       <c r="G19" s="6">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A20" s="40">
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C20" s="6" t="s">
         <v>28</v>
@@ -1720,11 +1732,11 @@
         <v>45559</v>
       </c>
       <c r="G20" s="6">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A21" s="40">
         <f t="shared" si="0"/>
         <v>12</v>
@@ -1745,11 +1757,11 @@
         <v>45609</v>
       </c>
       <c r="G21" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>-19</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A22" s="40">
         <f t="shared" si="0"/>
         <v>13</v>
@@ -1770,11 +1782,11 @@
         <v>45628</v>
       </c>
       <c r="G22" s="6">
-        <f t="shared" ref="G22:G41" si="2">IF(AND(E22&gt;0,F22&gt;0),F22-E22,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
+        <f t="shared" ref="G22:G41" si="3">IF(AND(E22&gt;0,F22&gt;0),F22-E22,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A23" s="40">
         <f t="shared" si="0"/>
         <v>14</v>
@@ -1795,11 +1807,11 @@
         <v>45628</v>
       </c>
       <c r="G23" s="6">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A24" s="40">
         <f t="shared" si="0"/>
         <v>15</v>
@@ -1820,11 +1832,11 @@
         <v>45628</v>
       </c>
       <c r="G24" s="6">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A25" s="40">
         <f t="shared" si="0"/>
         <v>16</v>
@@ -1845,11 +1857,11 @@
         <v>45628</v>
       </c>
       <c r="G25" s="6">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="40">
         <f t="shared" si="0"/>
         <v>17</v>
@@ -1870,11 +1882,11 @@
         <v>45628</v>
       </c>
       <c r="G26" s="6">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8" s="14" customFormat="1" ht="15.6" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" s="14" customFormat="1" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A27" s="41">
         <f t="shared" si="0"/>
         <v>18</v>
@@ -1891,16 +1903,16 @@
       <c r="E27" s="11">
         <v>45628</v>
       </c>
-      <c r="F27" s="11">
+      <c r="F27" s="88">
         <v>45628</v>
       </c>
       <c r="G27" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="H27" s="64"/>
     </row>
-    <row r="28" spans="1:8" s="17" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:8" s="17" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="42">
         <f>IF(D28=D27,A27+1,(D28*100))</f>
         <v>0</v>
@@ -1921,16 +1933,16 @@
         <v>45587</v>
       </c>
       <c r="G28" s="19">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>14</v>
       </c>
       <c r="H28" s="65" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A29" s="43">
-        <f t="shared" ref="A29:A39" si="3">IF(D29=D28,A28+1,(D29*100))</f>
+        <f t="shared" ref="A29:A39" si="4">IF(D29=D28,A28+1,(D29*100))</f>
         <v>1</v>
       </c>
       <c r="B29" s="5" t="s">
@@ -1949,16 +1961,16 @@
         <v>45553</v>
       </c>
       <c r="G29" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-20</v>
       </c>
       <c r="H29" s="86" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A30" s="43">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>2</v>
       </c>
       <c r="B30" s="5" t="s">
@@ -1977,14 +1989,14 @@
         <v>45553</v>
       </c>
       <c r="G30" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-20</v>
       </c>
       <c r="H30" s="87"/>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A31" s="43">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>3</v>
       </c>
       <c r="B31" s="5" t="s">
@@ -2003,14 +2015,14 @@
         <v>45553</v>
       </c>
       <c r="G31" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-20</v>
       </c>
       <c r="H31" s="87"/>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A32" s="43">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>4</v>
       </c>
       <c r="B32" s="5" t="s">
@@ -2029,14 +2041,14 @@
         <v>45553</v>
       </c>
       <c r="G32" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-20</v>
       </c>
       <c r="H32" s="87"/>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A33" s="43">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>5</v>
       </c>
       <c r="B33" s="5" t="s">
@@ -2055,18 +2067,18 @@
         <v>45553</v>
       </c>
       <c r="G33" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-20</v>
       </c>
       <c r="H33" s="87"/>
     </row>
-    <row r="34" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A34" s="43">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>6</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="C34" s="6" t="s">
         <v>33</v>
@@ -2081,20 +2093,20 @@
         <v>45583</v>
       </c>
       <c r="G34" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>10</v>
       </c>
       <c r="H34" s="66" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A35" s="43">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>7</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="C35" s="6" t="s">
         <v>34</v>
@@ -2109,20 +2121,18 @@
         <v>45564</v>
       </c>
       <c r="G35" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-9</v>
       </c>
-      <c r="H35" s="66" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="H35" s="66"/>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A36" s="43">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>8</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="C36" s="6" t="s">
         <v>35</v>
@@ -2137,20 +2147,20 @@
         <v>45564</v>
       </c>
       <c r="G36" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-9</v>
       </c>
       <c r="H36" s="63" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A37" s="43">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>9</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C37" s="27" t="s">
         <v>34</v>
@@ -2165,20 +2175,20 @@
         <v>45564</v>
       </c>
       <c r="G37" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-9</v>
       </c>
       <c r="H37" s="67" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.3">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A38" s="43">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>10</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C38" s="6" t="s">
         <v>35</v>
@@ -2193,16 +2203,16 @@
         <v>45562</v>
       </c>
       <c r="G38" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-11</v>
       </c>
       <c r="H38" s="63" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="39" spans="1:8" s="14" customFormat="1" ht="15.6" thickBot="1" x14ac:dyDescent="0.35">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" s="14" customFormat="1" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A39" s="44">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>11</v>
       </c>
       <c r="B39" s="9" t="s">
@@ -2221,20 +2231,20 @@
         <v>45562</v>
       </c>
       <c r="G39" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-11</v>
       </c>
       <c r="H39" s="64" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="40" spans="1:8" s="33" customFormat="1" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" s="33" customFormat="1" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A40" s="45">
         <f>IF(D40=D38,A38+1,(D40*100))</f>
         <v>100</v>
       </c>
       <c r="B40" s="28" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="C40" s="16" t="s">
         <v>28</v>
@@ -2246,20 +2256,20 @@
         <v>45579</v>
       </c>
       <c r="F40" s="31" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="G40" s="32"/>
       <c r="H40" s="68" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="41" spans="1:8" s="17" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:8" s="17" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="42">
         <f>IF(D41=D39,A39+1,(D41*100))</f>
         <v>100</v>
       </c>
       <c r="B41" s="15" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="C41" s="16" t="s">
         <v>28</v>
@@ -2274,14 +2284,14 @@
         <v>45596</v>
       </c>
       <c r="G41" s="19">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="H41" s="69"/>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A42" s="35">
-        <f t="shared" ref="A42:A63" si="4">IF(B42="","",IF(D42=D41,A41+1,(D42*100)))</f>
+        <f t="shared" ref="A42:A63" si="5">IF(B42="","",IF(D42=D41,A41+1,(D42*100)))</f>
         <v>101</v>
       </c>
       <c r="B42" s="5" t="s">
@@ -2300,13 +2310,13 @@
         <v>45600</v>
       </c>
       <c r="G42" s="6">
-        <f t="shared" ref="G42:G90" si="5">IF(B42="","",IF(AND(E42&gt;0,F42&gt;0),F42-E42,0))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+        <f t="shared" ref="G42:G91" si="6">IF(B42="","",IF(AND(E42&gt;0,F42&gt;0),F42-E42,0))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A43" s="43">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>102</v>
       </c>
       <c r="B43" s="5" t="s">
@@ -2325,13 +2335,13 @@
         <v>45593</v>
       </c>
       <c r="G43" s="6">
+        <f t="shared" si="6"/>
+        <v>-45</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A44" s="43">
         <f t="shared" si="5"/>
-        <v>-45</v>
-      </c>
-    </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A44" s="43">
-        <f t="shared" si="4"/>
         <v>103</v>
       </c>
       <c r="B44" s="5" t="s">
@@ -2351,16 +2361,16 @@
         <v>45562</v>
       </c>
       <c r="G44" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>-34</v>
       </c>
       <c r="H44" s="63" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A45" s="43">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>104</v>
       </c>
       <c r="B45" s="5" t="s">
@@ -2379,13 +2389,13 @@
         <v>45592</v>
       </c>
       <c r="G45" s="6">
+        <f t="shared" si="6"/>
+        <v>-4</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A46" s="43">
         <f t="shared" si="5"/>
-        <v>-4</v>
-      </c>
-    </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A46" s="43">
-        <f t="shared" si="4"/>
         <v>105</v>
       </c>
       <c r="B46" s="5" t="s">
@@ -2404,17 +2414,17 @@
         <v>45595</v>
       </c>
       <c r="G46" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>-1</v>
       </c>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A47" s="35">
         <f>IF(B47="","",IF(D47=D46,A46+1,(D47*100)))</f>
         <v>106</v>
       </c>
       <c r="B47" s="5" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="C47" s="6" t="s">
         <v>35</v>
@@ -2429,16 +2439,16 @@
         <v>45600</v>
       </c>
       <c r="G47" s="6">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="48" spans="1:8" ht="19.05" customHeight="1" x14ac:dyDescent="0.3">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="35" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="B48" s="5" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="C48" s="6" t="s">
         <v>35</v>
@@ -2457,7 +2467,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:8" ht="19.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:8" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="35">
         <f>IF(B49="","",IF(D49=Sheet1!D48,Sheet1!A48+1,(D49*100)))</f>
         <v>110.00000000000001</v>
@@ -2483,10 +2493,10 @@
         <v>-3</v>
       </c>
       <c r="H49" s="63" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="50" spans="1:8" s="54" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" s="54" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="49">
         <f>IF(B50="","",IF(D50=D47,A47+1,(D50*100)))</f>
         <v>200</v>
@@ -2508,18 +2518,18 @@
         <v>45611</v>
       </c>
       <c r="G50" s="53">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>3</v>
       </c>
       <c r="H50" s="70"/>
     </row>
-    <row r="51" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A51" s="35">
         <f>IF(B51="","",IF(D51=D48,A48+1,(D51*100)))</f>
         <v>200</v>
       </c>
       <c r="B51" s="5" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="C51" s="6" t="s">
         <v>33</v>
@@ -2534,17 +2544,17 @@
         <v>45607</v>
       </c>
       <c r="G51" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
     </row>
-    <row r="52" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A52" s="35">
         <f>IF(B52="","",IF(D52=D57,A57+1,(D52*100)))</f>
         <v>202</v>
       </c>
       <c r="B52" s="5" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="C52" s="6" t="s">
         <v>34</v>
@@ -2560,47 +2570,47 @@
         <v>45610</v>
       </c>
       <c r="G52" s="6">
+        <f t="shared" si="6"/>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A53" s="35">
         <f t="shared" si="5"/>
-        <v>4</v>
-      </c>
-    </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A53" s="35">
-        <f t="shared" si="4"/>
         <v>203</v>
       </c>
       <c r="B53" s="5" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="C53" s="6" t="s">
         <v>33</v>
       </c>
       <c r="D53" s="6">
-        <f t="shared" ref="D53:D98" si="6">IF(B53="","",D52)</f>
+        <f t="shared" ref="D53:D106" si="7">IF(B53="","",D52)</f>
         <v>2</v>
       </c>
       <c r="E53" s="85" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="F53" s="85"/>
       <c r="G53" s="85"/>
       <c r="H53" s="63" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="54" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A54" s="35">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>204</v>
       </c>
       <c r="B54" s="5" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="C54" s="6" t="s">
         <v>35</v>
       </c>
       <c r="D54" s="6">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>2</v>
       </c>
       <c r="E54" s="34">
@@ -2610,17 +2620,17 @@
         <v>45609</v>
       </c>
       <c r="G54" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>3</v>
       </c>
     </row>
-    <row r="55" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A55" s="35">
         <f>IF(B55="","",IF(D55=D60,A60+1,(D55*100)))</f>
         <v>207</v>
       </c>
       <c r="B55" s="5" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="C55" s="6" t="s">
         <v>33</v>
@@ -2636,23 +2646,23 @@
         <v>45605</v>
       </c>
       <c r="G55" s="6">
-        <f t="shared" ref="G55:G56" si="7">IF(B55="","",IF(AND(E55&gt;0,F55&gt;0),F55-E55,0))</f>
+        <f t="shared" ref="G55:G56" si="8">IF(B55="","",IF(AND(E55&gt;0,F55&gt;0),F55-E55,0))</f>
         <v>-1</v>
       </c>
     </row>
-    <row r="56" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A56" s="35">
         <f>IF(B56="","",IF(D56=D55,A55+1,(D56*100)))</f>
         <v>208</v>
       </c>
       <c r="B56" s="5" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="C56" s="6" t="s">
         <v>33</v>
       </c>
       <c r="D56" s="6">
-        <f t="shared" ref="D56" si="8">IF(B56="","",D55)</f>
+        <f t="shared" ref="D56" si="9">IF(B56="","",D55)</f>
         <v>2</v>
       </c>
       <c r="E56" s="34">
@@ -2662,17 +2672,17 @@
         <v>45607</v>
       </c>
       <c r="G56" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
     </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A57" s="35">
         <f>IF(B57="","",IF(D57=D51,A51+1,(D57*100)))</f>
         <v>201</v>
       </c>
       <c r="B57" s="5" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="C57" s="6" t="s">
         <v>34</v>
@@ -2681,45 +2691,45 @@
         <v>2</v>
       </c>
       <c r="E57" s="85" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="F57" s="85"/>
       <c r="G57" s="85"/>
       <c r="H57" s="63" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.3">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A58" s="35">
         <f>IF(B58="","",IF(D58=D56,A56+1,(D58*100)))</f>
         <v>209</v>
       </c>
       <c r="B58" s="5" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="C58" s="6" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="D58" s="6">
         <f>IF(B58="","",D56)</f>
         <v>2</v>
       </c>
       <c r="E58" s="85" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="F58" s="85"/>
       <c r="G58" s="85"/>
       <c r="H58" s="63" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.3">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A59" s="35">
         <f>IF(B59="","",IF(D59=D54,A54+1,(D59*100)))</f>
         <v>205</v>
       </c>
       <c r="B59" s="5" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="C59" s="6" t="s">
         <v>34</v>
@@ -2729,18 +2739,18 @@
         <v>2</v>
       </c>
       <c r="E59" s="85" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="F59" s="85"/>
       <c r="G59" s="85"/>
     </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A60" s="35">
         <f>IF(B60="","",IF(D60=D59,A59+1,(D60*100)))</f>
         <v>206</v>
       </c>
       <c r="B60" s="5" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="C60" s="6" t="s">
         <v>33</v>
@@ -2750,21 +2760,21 @@
         <v>2</v>
       </c>
       <c r="E60" s="85" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="F60" s="85"/>
       <c r="G60" s="85"/>
       <c r="H60" s="63" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="61" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A61" s="35">
         <f>IF(B61="","",IF(D61=D58,A58+1,(D61*100)))</f>
         <v>210</v>
       </c>
       <c r="B61" s="5" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="C61" s="6" t="s">
         <v>34</v>
@@ -2784,13 +2794,13 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="62" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A62" s="35">
         <f>IF(B62="","",IF(D62=D60,A60+1,(D62*100)))</f>
         <v>207</v>
       </c>
       <c r="B62" s="5" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="C62" s="6" t="s">
         <v>34</v>
@@ -2807,13 +2817,13 @@
         <v>45607</v>
       </c>
       <c r="G62" s="6">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="63" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A63" s="35">
         <f t="shared" si="5"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="63" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A63" s="35">
-        <f t="shared" si="4"/>
         <v>208</v>
       </c>
       <c r="B63" s="5" t="s">
@@ -2823,49 +2833,49 @@
         <v>34</v>
       </c>
       <c r="D63" s="6">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>2</v>
       </c>
       <c r="E63" s="34">
-        <f t="shared" ref="E63:E77" si="9">IF(B63="","",IF(D63=D62,E62,E62+14))</f>
+        <f t="shared" ref="E63:E77" si="10">IF(B63="","",IF(D63=D62,E62,E62+14))</f>
         <v>45606</v>
       </c>
       <c r="F63" s="11">
         <v>45607</v>
       </c>
       <c r="G63" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
     </row>
-    <row r="64" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A64" s="35">
-        <f t="shared" ref="A64" si="10">IF(B64="","",IF(D64=D63,A63+1,(D64*100)))</f>
+        <f t="shared" ref="A64" si="11">IF(B64="","",IF(D64=D63,A63+1,(D64*100)))</f>
         <v>209</v>
       </c>
       <c r="B64" s="5" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="C64" s="6" t="s">
         <v>35</v>
       </c>
       <c r="D64" s="6">
-        <f t="shared" ref="D64" si="11">IF(B64="","",D63)</f>
+        <f t="shared" ref="D64" si="12">IF(B64="","",D63)</f>
         <v>2</v>
       </c>
       <c r="E64" s="34">
-        <f t="shared" ref="E64" si="12">IF(B64="","",IF(D64=D63,E63,E63+14))</f>
+        <f t="shared" ref="E64" si="13">IF(B64="","",IF(D64=D63,E63,E63+14))</f>
         <v>45606</v>
       </c>
       <c r="F64" s="11">
         <v>45609</v>
       </c>
       <c r="G64" s="6">
-        <f t="shared" ref="G64" si="13">IF(B64="","",IF(AND(E64&gt;0,F64&gt;0),F64-E64,0))</f>
+        <f t="shared" ref="G64" si="14">IF(B64="","",IF(AND(E64&gt;0,F64&gt;0),F64-E64,0))</f>
         <v>3</v>
       </c>
     </row>
-    <row r="65" spans="1:8" ht="19.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:8" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" s="35">
         <f>IF(B65="","",IF(D65=Sheet1!D63,Sheet1!A63+1,(D65*100)))</f>
         <v>209</v>
@@ -2891,10 +2901,10 @@
         <v>4</v>
       </c>
       <c r="H65" s="63" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="66" spans="1:8" s="54" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="66" spans="1:8" s="54" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66" s="49">
         <f>IF(B66="","",IF(D66=D60,A60+1,(D66*100)))</f>
         <v>300</v>
@@ -2914,18 +2924,18 @@
       </c>
       <c r="F66" s="51"/>
       <c r="G66" s="6">
-        <f t="shared" ref="G66:G82" si="14">IF(AND(E66&gt;0,F66&gt;0),F66-E66,0)</f>
+        <f t="shared" ref="G66:G82" si="15">IF(AND(E66&gt;0,F66&gt;0),F66-E66,0)</f>
         <v>0</v>
       </c>
       <c r="H66" s="70"/>
     </row>
-    <row r="67" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A67" s="35">
         <f>IF(B67="","",IF(D67=D66,A66+1,(D67*100)))</f>
         <v>301</v>
       </c>
       <c r="B67" s="5" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="C67" s="6" t="s">
         <v>33</v>
@@ -2940,17 +2950,17 @@
         <v>45612</v>
       </c>
       <c r="G67" s="6">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>-1</v>
       </c>
     </row>
-    <row r="68" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A68" s="35">
-        <f t="shared" ref="A68:A98" si="15">IF(B68="","",IF(D68=D67,A67+1,(D68*100)))</f>
+        <f t="shared" ref="A68:A106" si="16">IF(B68="","",IF(D68=D67,A67+1,(D68*100)))</f>
         <v>302</v>
       </c>
       <c r="B68" s="5" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="C68" s="6" t="s">
         <v>33</v>
@@ -2965,17 +2975,17 @@
         <v>45612</v>
       </c>
       <c r="G68" s="6">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>-1</v>
       </c>
     </row>
-    <row r="69" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A69" s="35">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>303</v>
       </c>
       <c r="B69" s="5" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="C69" s="6" t="s">
         <v>33</v>
@@ -2990,17 +3000,17 @@
         <v>45610</v>
       </c>
       <c r="G69" s="6">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>-3</v>
       </c>
     </row>
-    <row r="70" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A70" s="35">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>304</v>
       </c>
       <c r="B70" s="5" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="C70" s="6" t="s">
         <v>33</v>
@@ -3015,17 +3025,17 @@
         <v>45612</v>
       </c>
       <c r="G70" s="6">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>-1</v>
       </c>
     </row>
-    <row r="71" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A71" s="35">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>305</v>
       </c>
       <c r="B71" s="5" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="C71" s="6" t="s">
         <v>33</v>
@@ -3040,20 +3050,17 @@
         <v>45606</v>
       </c>
       <c r="G71" s="6">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>-7</v>
       </c>
-      <c r="H71" s="63" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="72" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    </row>
+    <row r="72" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A72" s="35">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>306</v>
       </c>
       <c r="B72" s="5" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="C72" s="6" t="s">
         <v>33</v>
@@ -3068,17 +3075,17 @@
         <v>45613</v>
       </c>
       <c r="G72" s="6">
-        <f t="shared" si="14"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="73" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+        <f t="shared" si="15"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A73" s="35">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>307</v>
       </c>
       <c r="B73" s="5" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="C73" s="6" t="s">
         <v>34</v>
@@ -3093,17 +3100,17 @@
         <v>45616</v>
       </c>
       <c r="G73" s="6">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>3</v>
       </c>
     </row>
-    <row r="74" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A74" s="35">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>308</v>
       </c>
       <c r="B74" s="5" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="C74" s="6" t="s">
         <v>34</v>
@@ -3118,13 +3125,13 @@
         <v>45613</v>
       </c>
       <c r="G74" s="6">
-        <f t="shared" si="14"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="75" spans="1:8" ht="19.05" customHeight="1" x14ac:dyDescent="0.3">
+        <f t="shared" si="15"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75" spans="1:8" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A75" s="35">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>309</v>
       </c>
       <c r="B75" s="5" t="s">
@@ -3143,20 +3150,20 @@
         <v>45616</v>
       </c>
       <c r="G75" s="6">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>3</v>
       </c>
       <c r="H75" s="63" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="76" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="76" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A76" s="35">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>310</v>
       </c>
       <c r="B76" s="5" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="C76" s="6" t="s">
         <v>34</v>
@@ -3165,81 +3172,81 @@
         <v>3</v>
       </c>
       <c r="E76" s="34">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>45613</v>
       </c>
       <c r="F76" s="11">
         <v>45613</v>
       </c>
       <c r="G76" s="6">
-        <f t="shared" si="14"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="77" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+        <f t="shared" si="15"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A77" s="35">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>311</v>
       </c>
       <c r="B77" s="5" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="C77" s="6" t="s">
         <v>35</v>
       </c>
       <c r="D77" s="6">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>3</v>
       </c>
       <c r="E77" s="34">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>45613</v>
       </c>
       <c r="F77" s="11">
         <v>45616</v>
       </c>
       <c r="G77" s="6">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>3</v>
       </c>
     </row>
-    <row r="78" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A78" s="35">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>312</v>
       </c>
       <c r="B78" s="5" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="C78" s="6" t="s">
         <v>33</v>
       </c>
       <c r="D78" s="6">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>3</v>
       </c>
       <c r="E78" s="85" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="F78" s="85"/>
       <c r="G78" s="85"/>
       <c r="H78" s="63" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="79" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="79" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A79" s="35">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>313</v>
       </c>
       <c r="B79" s="5" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="C79" s="6" t="s">
         <v>34</v>
       </c>
       <c r="D79" s="6">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>3</v>
       </c>
       <c r="E79" s="34">
@@ -3253,16 +3260,16 @@
         <v>1</v>
       </c>
       <c r="H79" s="63" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="80" spans="1:8" x14ac:dyDescent="0.3">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="80" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A80" s="35">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>314</v>
       </c>
       <c r="B80" s="5" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="C80" s="6" t="s">
         <v>34</v>
@@ -3271,24 +3278,24 @@
         <v>3</v>
       </c>
       <c r="E80" s="85" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="F80" s="85"/>
       <c r="G80" s="85"/>
     </row>
-    <row r="81" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A81" s="35">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>315</v>
       </c>
       <c r="B81" s="5" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="C81" s="6" t="s">
         <v>35</v>
       </c>
       <c r="D81" s="6">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>3</v>
       </c>
       <c r="E81" s="34">
@@ -3298,13 +3305,13 @@
         <v>45616</v>
       </c>
       <c r="G81" s="6">
-        <f t="shared" si="14"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="82" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+        <f t="shared" si="15"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A82" s="35">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>316</v>
       </c>
       <c r="B82" s="5" t="str">
@@ -3324,13 +3331,13 @@
         <v>45616</v>
       </c>
       <c r="G82" s="6">
-        <f t="shared" si="14"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="83" spans="1:8" s="54" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+        <f t="shared" si="15"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83" spans="1:8" s="54" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A83" s="35">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>400</v>
       </c>
       <c r="B83" s="50" t="str">
@@ -3350,18 +3357,18 @@
         <v>45628</v>
       </c>
       <c r="G83" s="6">
-        <f t="shared" ref="G83" si="16">IF(AND(E83&gt;0,F83&gt;0),F83-E83,0)</f>
+        <f t="shared" ref="G83" si="17">IF(AND(E83&gt;0,F83&gt;0),F83-E83,0)</f>
         <v>0</v>
       </c>
       <c r="H83" s="70"/>
     </row>
-    <row r="84" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A84" s="35">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>401</v>
       </c>
-      <c r="B84" s="71" t="s">
-        <v>124</v>
+      <c r="B84" s="5" t="s">
+        <v>107</v>
       </c>
       <c r="C84" s="6" t="s">
         <v>33</v>
@@ -3372,53 +3379,49 @@
       <c r="E84" s="34">
         <v>45625</v>
       </c>
-      <c r="F84" s="11">
-        <v>45620</v>
-      </c>
       <c r="G84" s="6">
-        <f t="shared" si="5"/>
-        <v>-5</v>
-      </c>
-    </row>
-    <row r="85" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="85" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A85" s="35">
-        <f>IF(B85="","",IF(D85=D90,A90+1,(D85*100)))</f>
-        <v>406</v>
-      </c>
-      <c r="B85" s="5" t="s">
-        <v>118</v>
+        <f t="shared" si="16"/>
+        <v>402</v>
+      </c>
+      <c r="B85" s="71" t="s">
+        <v>116</v>
       </c>
       <c r="C85" s="6" t="s">
         <v>33</v>
       </c>
       <c r="D85" s="6">
-        <f>IF(B85="","",D90)</f>
         <v>4</v>
       </c>
       <c r="E85" s="34">
-        <v>45628</v>
+        <v>45625</v>
       </c>
       <c r="F85" s="11">
-        <v>45622</v>
+        <v>45620</v>
       </c>
       <c r="G85" s="6">
-        <f>IF(B85="","",IF(AND(E85&gt;0,F85&gt;0),F85-E85,0))</f>
-        <v>-6</v>
-      </c>
-    </row>
-    <row r="86" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+        <f t="shared" si="6"/>
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="86" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A86" s="35">
-        <f>IF(B86="","",IF(D86=D85,A85+1,(D86*100)))</f>
+        <f>IF(B86="","",IF(D86=D91,A91+1,(D86*100)))</f>
         <v>407</v>
       </c>
       <c r="B86" s="5" t="s">
-        <v>119</v>
+        <v>110</v>
       </c>
       <c r="C86" s="6" t="s">
         <v>33</v>
       </c>
       <c r="D86" s="6">
-        <f>IF(B86="","",D85)</f>
+        <f>IF(B86="","",D91)</f>
         <v>4</v>
       </c>
       <c r="E86" s="34">
@@ -3432,44 +3435,44 @@
         <v>-6</v>
       </c>
     </row>
-    <row r="87" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A87" s="35">
-        <f>IF(B87="","",IF(D87=D84,A84+1,(D87*100)))</f>
-        <v>402</v>
+        <f>IF(B87="","",IF(D87=D86,A86+1,(D87*100)))</f>
+        <v>408</v>
       </c>
       <c r="B87" s="5" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="C87" s="6" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D87" s="6">
+        <f>IF(B87="","",D86)</f>
         <v>4</v>
       </c>
       <c r="E87" s="34">
-        <v>45625</v>
+        <v>45628</v>
       </c>
       <c r="F87" s="11">
-        <v>45618</v>
+        <v>45622</v>
       </c>
       <c r="G87" s="6">
-        <f t="shared" si="5"/>
-        <v>-7</v>
-      </c>
-    </row>
-    <row r="88" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+        <f>IF(B87="","",IF(AND(E87&gt;0,F87&gt;0),F87-E87,0))</f>
+        <v>-6</v>
+      </c>
+    </row>
+    <row r="88" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A88" s="35">
-        <f t="shared" si="15"/>
+        <f>IF(B88="","",IF(D88=D85,A85+1,(D88*100)))</f>
         <v>403</v>
       </c>
       <c r="B88" s="5" t="s">
-        <v>116</v>
+        <v>109</v>
       </c>
       <c r="C88" s="6" t="s">
         <v>34</v>
       </c>
       <c r="D88" s="6">
-        <f t="shared" si="6"/>
         <v>4</v>
       </c>
       <c r="E88" s="34">
@@ -3479,23 +3482,23 @@
         <v>45618</v>
       </c>
       <c r="G88" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>-7</v>
       </c>
     </row>
-    <row r="89" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A89" s="35">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>404</v>
       </c>
       <c r="B89" s="5" t="s">
-        <v>98</v>
+        <v>108</v>
       </c>
       <c r="C89" s="6" t="s">
         <v>34</v>
       </c>
       <c r="D89" s="6">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>4</v>
       </c>
       <c r="E89" s="34">
@@ -3505,368 +3508,443 @@
         <v>45618</v>
       </c>
       <c r="G89" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>-7</v>
       </c>
     </row>
-    <row r="90" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A90" s="35">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>405</v>
       </c>
       <c r="B90" s="5" t="s">
-        <v>114</v>
+        <v>94</v>
       </c>
       <c r="C90" s="6" t="s">
         <v>34</v>
       </c>
       <c r="D90" s="6">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>4</v>
       </c>
       <c r="E90" s="34">
         <v>45625</v>
       </c>
       <c r="F90" s="11">
-        <v>45618</v>
+        <v>45620</v>
       </c>
       <c r="G90" s="6">
-        <f t="shared" si="5"/>
-        <v>-7</v>
-      </c>
-    </row>
-    <row r="91" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+        <f t="shared" si="6"/>
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="91" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A91" s="35">
-        <f>IF(B91="","",IF(D91=D86,A86+1,(D91*100)))</f>
-        <v>408</v>
+        <f t="shared" si="16"/>
+        <v>406</v>
       </c>
       <c r="B91" s="5" t="s">
-        <v>120</v>
+        <v>106</v>
       </c>
       <c r="C91" s="6" t="s">
         <v>34</v>
       </c>
       <c r="D91" s="6">
-        <f>IF(B91="","",D86)</f>
+        <f t="shared" si="7"/>
         <v>4</v>
       </c>
       <c r="E91" s="34">
-        <v>45628</v>
+        <v>45625</v>
       </c>
       <c r="F91" s="11">
         <v>45618</v>
       </c>
       <c r="G91" s="6">
-        <f>IF(B91="","",IF(AND(E91&gt;0,F91&gt;0),F91-E91,0))</f>
-        <v>-10</v>
-      </c>
-    </row>
-    <row r="92" spans="1:8" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A92" s="76" t="s">
-        <v>125</v>
-      </c>
-      <c r="B92" s="76"/>
-      <c r="C92" s="76"/>
-      <c r="D92" s="76"/>
-      <c r="E92" s="76"/>
-      <c r="F92" s="76"/>
-      <c r="G92" s="76"/>
-    </row>
-    <row r="93" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A93" s="35">
-        <f>IF(B93="","",IF(D93=D91,A91+1,(D93*100)))</f>
+        <f t="shared" si="6"/>
+        <v>-7</v>
+      </c>
+    </row>
+    <row r="92" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A92" s="35">
+        <f>IF(B92="","",IF(D92=D87,A87+1,(D92*100)))</f>
         <v>409</v>
       </c>
-      <c r="B93" s="5" t="s">
-        <v>123</v>
-      </c>
-      <c r="C93" s="6" t="s">
+      <c r="B92" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="C92" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="D92" s="6">
+        <f>IF(B92="","",D87)</f>
+        <v>4</v>
+      </c>
+      <c r="E92" s="34">
+        <v>45628</v>
+      </c>
+      <c r="F92" s="11">
+        <v>45620</v>
+      </c>
+      <c r="G92" s="6">
+        <f>IF(B92="","",IF(AND(E92&gt;0,F92&gt;0),F92-E92,0))</f>
+        <v>-8</v>
+      </c>
+    </row>
+    <row r="93" spans="1:8" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A93" s="76" t="s">
+        <v>117</v>
+      </c>
+      <c r="B93" s="76"/>
+      <c r="C93" s="76"/>
+      <c r="D93" s="76"/>
+      <c r="E93" s="76"/>
+      <c r="F93" s="76"/>
+      <c r="G93" s="76"/>
+    </row>
+    <row r="94" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A94" s="35">
+        <f>IF(B94="","",IF(D94=D92,A92+1,(D94*100)))</f>
+        <v>410</v>
+      </c>
+      <c r="B94" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="C94" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="D93" s="6">
-        <f>IF(B93="","",D91)</f>
+      <c r="D94" s="6">
+        <f>IF(B94="","",D92)</f>
         <v>4</v>
       </c>
-      <c r="E93" s="34">
-        <v>45628</v>
-      </c>
-      <c r="G93" s="6">
-        <f>IF(B93="","",IF(AND(E93&gt;0,F93&gt;0),F93-E93,0))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="94" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A94" s="35">
-        <f t="shared" ref="A94:A98" si="17">IF(B94="","",IF(D94=D92,A92+1,(D94*100)))</f>
-        <v>400</v>
-      </c>
-      <c r="B94" s="5" t="s">
+      <c r="E94" s="34">
+        <v>45628</v>
+      </c>
+      <c r="F94" s="11">
+        <v>45627</v>
+      </c>
+      <c r="G94" s="6">
+        <f>IF(B94="","",IF(AND(E94&gt;0,F94&gt;0),F94-E94,0))</f>
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="95" spans="1:8" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A95" s="35">
+        <f>IF(B95="","",IF(D95=D94,A94+1,(D95*100)))</f>
+        <v>411</v>
+      </c>
+      <c r="B95" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="C95" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="D95" s="6">
+        <f>IF(B95="","",D94)</f>
+        <v>4</v>
+      </c>
+      <c r="E95" s="34">
+        <v>45628</v>
+      </c>
+      <c r="G95" s="6">
+        <f t="shared" ref="G95:G143" si="18">IF(B95="","",IF(AND(E95&gt;0,F95&gt;0),F95-E95,0))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="96" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A96" s="35">
+        <f t="shared" si="16"/>
+        <v>412</v>
+      </c>
+      <c r="B96" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C96" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="D96" s="6">
+        <f t="shared" si="7"/>
+        <v>4</v>
+      </c>
+      <c r="E96" s="34">
+        <v>45628</v>
+      </c>
+      <c r="F96" s="11">
+        <v>45628</v>
+      </c>
+      <c r="G96" s="6">
+        <f t="shared" si="18"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="97" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A97" s="35">
+        <f t="shared" si="16"/>
+        <v>413</v>
+      </c>
+      <c r="B97" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="C97" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="D97" s="6">
+        <f t="shared" si="7"/>
+        <v>4</v>
+      </c>
+      <c r="E97" s="34">
+        <v>45628</v>
+      </c>
+      <c r="F97" s="11">
+        <v>45628</v>
+      </c>
+      <c r="G97" s="6">
+        <f t="shared" si="18"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="98" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A98" s="35">
+        <f t="shared" si="16"/>
+        <v>414</v>
+      </c>
+      <c r="B98" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="C98" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="D98" s="6">
+        <f t="shared" si="7"/>
+        <v>4</v>
+      </c>
+      <c r="E98" s="34">
+        <v>45628</v>
+      </c>
+      <c r="F98" s="11">
+        <v>45628</v>
+      </c>
+      <c r="G98" s="6">
+        <f t="shared" si="18"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="99" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A99" s="35">
+        <f t="shared" si="16"/>
+        <v>415</v>
+      </c>
+      <c r="B99" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="C99" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="D99" s="6">
+        <f t="shared" si="7"/>
+        <v>4</v>
+      </c>
+      <c r="E99" s="34">
+        <v>45628</v>
+      </c>
+      <c r="F99" s="11">
+        <v>45628</v>
+      </c>
+      <c r="G99" s="6">
+        <f t="shared" si="18"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="100" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A100" s="35">
+        <f t="shared" si="16"/>
+        <v>416</v>
+      </c>
+      <c r="B100" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="C100" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="D100" s="6">
+        <f t="shared" si="7"/>
+        <v>4</v>
+      </c>
+      <c r="E100" s="34">
+        <v>45628</v>
+      </c>
+      <c r="F100" s="11">
+        <v>45628</v>
+      </c>
+      <c r="G100" s="6">
+        <f t="shared" si="18"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="101" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A101" s="35">
+        <f t="shared" si="16"/>
+        <v>417</v>
+      </c>
+      <c r="B101" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="C94" s="6" t="s">
+      <c r="C101" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="D94" s="6">
+      <c r="D101" s="6">
+        <f t="shared" si="7"/>
         <v>4</v>
       </c>
-      <c r="E94" s="34">
-        <v>45628</v>
-      </c>
-      <c r="F94" s="11">
+      <c r="E101" s="34">
+        <v>45628</v>
+      </c>
+      <c r="F101" s="11">
         <f>F63</f>
         <v>45607</v>
       </c>
-      <c r="G94" s="6">
-        <f t="shared" ref="G94:G135" si="18">IF(B94="","",IF(AND(E94&gt;0,F94&gt;0),F94-E94,0))</f>
+      <c r="G101" s="6">
+        <f t="shared" si="18"/>
         <v>-21</v>
       </c>
     </row>
-    <row r="95" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A95" s="35">
-        <f t="shared" si="17"/>
-        <v>410</v>
-      </c>
-      <c r="B95" s="5" t="s">
-        <v>104</v>
-      </c>
-      <c r="C95" s="6" t="s">
+    <row r="102" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A102" s="35">
+        <f t="shared" si="16"/>
+        <v>418</v>
+      </c>
+      <c r="B102" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="C102" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="D95" s="6">
+      <c r="D102" s="6">
+        <f t="shared" si="7"/>
         <v>4</v>
       </c>
-      <c r="E95" s="34">
-        <v>45628</v>
-      </c>
-      <c r="G95" s="6">
+      <c r="E102" s="34">
+        <v>45628</v>
+      </c>
+      <c r="F102" s="11">
+        <v>45628</v>
+      </c>
+      <c r="G102" s="6">
         <f t="shared" si="18"/>
         <v>0</v>
       </c>
     </row>
-    <row r="96" spans="1:8" ht="30" x14ac:dyDescent="0.3">
-      <c r="A96" s="35">
-        <f t="shared" si="17"/>
-        <v>401</v>
-      </c>
-      <c r="B96" s="72" t="s">
-        <v>121</v>
-      </c>
-      <c r="C96" s="6" t="s">
+    <row r="103" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A103" s="35">
+        <f t="shared" si="16"/>
+        <v>419</v>
+      </c>
+      <c r="B103" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="C103" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="D103" s="6">
+        <f t="shared" si="7"/>
+        <v>4</v>
+      </c>
+      <c r="E103" s="34">
+        <v>45628</v>
+      </c>
+      <c r="G103" s="6">
+        <f t="shared" si="18"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="104" spans="1:7" ht="34" x14ac:dyDescent="0.2">
+      <c r="A104" s="35">
+        <f t="shared" si="16"/>
+        <v>420</v>
+      </c>
+      <c r="B104" s="72" t="s">
+        <v>113</v>
+      </c>
+      <c r="C104" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="D96" s="6">
+      <c r="D104" s="6">
+        <f t="shared" si="7"/>
         <v>4</v>
       </c>
-      <c r="E96" s="34">
-        <v>45628</v>
-      </c>
-      <c r="G96" s="6">
-        <f>IF(B96="","",IF(AND(E96&gt;0,F96&gt;0),F96-E96,0))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="97" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A97" s="35">
-        <f t="shared" si="17"/>
-        <v>411</v>
-      </c>
-      <c r="B97" s="5" t="s">
-        <v>122</v>
-      </c>
-      <c r="C97" s="6" t="s">
+      <c r="E104" s="34">
+        <v>45628</v>
+      </c>
+      <c r="F104" s="11">
+        <v>45627</v>
+      </c>
+      <c r="G104" s="6">
+        <f>IF(B104="","",IF(AND(E104&gt;0,F104&gt;0),F104-E104,0))</f>
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="105" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A105" s="35">
+        <f t="shared" si="16"/>
+        <v>421</v>
+      </c>
+      <c r="B105" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="C105" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="D97" s="6">
+      <c r="D105" s="6">
+        <f t="shared" si="7"/>
         <v>4</v>
       </c>
-      <c r="E97" s="34">
-        <v>45628</v>
-      </c>
-      <c r="G97" s="6">
-        <f>IF(B97="","",IF(AND(E97&gt;0,F97&gt;0),F97-E97,0))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="98" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A98" s="35">
-        <f t="shared" si="17"/>
-        <v>402</v>
-      </c>
-      <c r="B98" s="5" t="s">
-        <v>103</v>
-      </c>
-      <c r="C98" s="6" t="s">
+      <c r="E105" s="34">
+        <v>45628</v>
+      </c>
+      <c r="F105" s="88">
+        <v>45627</v>
+      </c>
+      <c r="G105" s="6">
+        <f>IF(B105="","",IF(AND(E105&gt;0,F105&gt;0),F105-E105,0))</f>
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="106" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A106" s="35">
+        <f t="shared" si="16"/>
+        <v>422</v>
+      </c>
+      <c r="B106" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C106" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="D98" s="6">
+      <c r="D106" s="6">
+        <f t="shared" si="7"/>
         <v>4</v>
       </c>
-      <c r="E98" s="34">
+      <c r="E106" s="34">
         <v>45629</v>
       </c>
-      <c r="F98" s="11">
+      <c r="F106" s="11">
         <v>45629</v>
       </c>
-      <c r="G98" s="6">
-        <f>IF(B98="","",IF(AND(E98&gt;0,F98&gt;0),F98-E98,0))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="99" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A99" s="35" t="str">
-        <f>IF(B99="","",IF(D99=#REF!,#REF!+1,(D99*100)))</f>
-        <v/>
-      </c>
-      <c r="D99" s="6" t="str">
-        <f>IF(B99="","",#REF!)</f>
-        <v/>
-      </c>
-      <c r="E99" s="34" t="str">
-        <f>IF(B99="","",IF(D99=#REF!,#REF!,#REF!+14))</f>
-        <v/>
-      </c>
-      <c r="G99" s="6" t="str">
-        <f t="shared" si="18"/>
-        <v/>
-      </c>
-    </row>
-    <row r="100" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A100" s="35" t="str">
-        <f t="shared" ref="A100:A135" si="19">IF(B100="","",IF(D100=D99,A99+1,(D100*100)))</f>
-        <v/>
-      </c>
-      <c r="D100" s="6" t="str">
-        <f t="shared" ref="D100:D135" si="20">IF(B100="","",D99)</f>
-        <v/>
-      </c>
-      <c r="E100" s="34" t="str">
-        <f t="shared" ref="E100:E135" si="21">IF(B100="","",IF(D100=D99,E99,E99+14))</f>
-        <v/>
-      </c>
-      <c r="G100" s="6" t="str">
-        <f t="shared" si="18"/>
-        <v/>
-      </c>
-    </row>
-    <row r="101" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A101" s="35" t="str">
-        <f t="shared" si="19"/>
-        <v/>
-      </c>
-      <c r="D101" s="6" t="str">
-        <f t="shared" si="20"/>
-        <v/>
-      </c>
-      <c r="E101" s="34" t="str">
-        <f t="shared" si="21"/>
-        <v/>
-      </c>
-      <c r="G101" s="6" t="str">
-        <f t="shared" si="18"/>
-        <v/>
-      </c>
-    </row>
-    <row r="102" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A102" s="35" t="str">
-        <f t="shared" si="19"/>
-        <v/>
-      </c>
-      <c r="D102" s="6" t="str">
-        <f t="shared" si="20"/>
-        <v/>
-      </c>
-      <c r="E102" s="34" t="str">
-        <f t="shared" si="21"/>
-        <v/>
-      </c>
-      <c r="G102" s="6" t="str">
-        <f t="shared" si="18"/>
-        <v/>
-      </c>
-    </row>
-    <row r="103" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A103" s="35" t="str">
-        <f t="shared" si="19"/>
-        <v/>
-      </c>
-      <c r="D103" s="6" t="str">
-        <f t="shared" si="20"/>
-        <v/>
-      </c>
-      <c r="E103" s="34" t="str">
-        <f t="shared" si="21"/>
-        <v/>
-      </c>
-      <c r="G103" s="6" t="str">
-        <f t="shared" si="18"/>
-        <v/>
-      </c>
-    </row>
-    <row r="104" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A104" s="35" t="str">
-        <f t="shared" si="19"/>
-        <v/>
-      </c>
-      <c r="D104" s="6" t="str">
-        <f t="shared" si="20"/>
-        <v/>
-      </c>
-      <c r="E104" s="34" t="str">
-        <f t="shared" si="21"/>
-        <v/>
-      </c>
-      <c r="G104" s="6" t="str">
-        <f t="shared" si="18"/>
-        <v/>
-      </c>
-    </row>
-    <row r="105" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A105" s="35" t="str">
-        <f t="shared" si="19"/>
-        <v/>
-      </c>
-      <c r="D105" s="6" t="str">
-        <f t="shared" si="20"/>
-        <v/>
-      </c>
-      <c r="E105" s="34" t="str">
-        <f t="shared" si="21"/>
-        <v/>
-      </c>
-      <c r="G105" s="6" t="str">
-        <f t="shared" si="18"/>
-        <v/>
-      </c>
-    </row>
-    <row r="106" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A106" s="35" t="str">
-        <f t="shared" si="19"/>
-        <v/>
-      </c>
-      <c r="D106" s="6" t="str">
-        <f t="shared" si="20"/>
-        <v/>
-      </c>
-      <c r="E106" s="34" t="str">
-        <f t="shared" si="21"/>
-        <v/>
-      </c>
-      <c r="G106" s="6" t="str">
-        <f t="shared" si="18"/>
-        <v/>
-      </c>
-    </row>
-    <row r="107" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G106" s="6">
+        <f>IF(B106="","",IF(AND(E106&gt;0,F106&gt;0),F106-E106,0))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="107" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A107" s="35" t="str">
-        <f t="shared" si="19"/>
+        <f>IF(B107="","",IF(D107=#REF!,#REF!+1,(D107*100)))</f>
         <v/>
       </c>
       <c r="D107" s="6" t="str">
-        <f t="shared" si="20"/>
+        <f>IF(B107="","",#REF!)</f>
         <v/>
       </c>
       <c r="E107" s="34" t="str">
-        <f t="shared" si="21"/>
+        <f>IF(B107="","",IF(D107=#REF!,#REF!,#REF!+14))</f>
         <v/>
       </c>
       <c r="G107" s="6" t="str">
@@ -3874,17 +3952,17 @@
         <v/>
       </c>
     </row>
-    <row r="108" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A108" s="35" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" ref="A108:A143" si="19">IF(B108="","",IF(D108=D107,A107+1,(D108*100)))</f>
         <v/>
       </c>
       <c r="D108" s="6" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" ref="D108:D143" si="20">IF(B108="","",D107)</f>
         <v/>
       </c>
       <c r="E108" s="34" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" ref="E108:E143" si="21">IF(B108="","",IF(D108=D107,E107,E107+14))</f>
         <v/>
       </c>
       <c r="G108" s="6" t="str">
@@ -3892,7 +3970,7 @@
         <v/>
       </c>
     </row>
-    <row r="109" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A109" s="35" t="str">
         <f t="shared" si="19"/>
         <v/>
@@ -3910,7 +3988,7 @@
         <v/>
       </c>
     </row>
-    <row r="110" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A110" s="35" t="str">
         <f t="shared" si="19"/>
         <v/>
@@ -3928,7 +4006,7 @@
         <v/>
       </c>
     </row>
-    <row r="111" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A111" s="35" t="str">
         <f t="shared" si="19"/>
         <v/>
@@ -3946,7 +4024,7 @@
         <v/>
       </c>
     </row>
-    <row r="112" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A112" s="35" t="str">
         <f t="shared" si="19"/>
         <v/>
@@ -3964,7 +4042,7 @@
         <v/>
       </c>
     </row>
-    <row r="113" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A113" s="35" t="str">
         <f t="shared" si="19"/>
         <v/>
@@ -3982,7 +4060,7 @@
         <v/>
       </c>
     </row>
-    <row r="114" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A114" s="35" t="str">
         <f t="shared" si="19"/>
         <v/>
@@ -4000,7 +4078,7 @@
         <v/>
       </c>
     </row>
-    <row r="115" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A115" s="35" t="str">
         <f t="shared" si="19"/>
         <v/>
@@ -4018,7 +4096,7 @@
         <v/>
       </c>
     </row>
-    <row r="116" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A116" s="35" t="str">
         <f t="shared" si="19"/>
         <v/>
@@ -4036,7 +4114,7 @@
         <v/>
       </c>
     </row>
-    <row r="117" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A117" s="35" t="str">
         <f t="shared" si="19"/>
         <v/>
@@ -4054,7 +4132,7 @@
         <v/>
       </c>
     </row>
-    <row r="118" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A118" s="35" t="str">
         <f t="shared" si="19"/>
         <v/>
@@ -4072,7 +4150,7 @@
         <v/>
       </c>
     </row>
-    <row r="119" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A119" s="35" t="str">
         <f t="shared" si="19"/>
         <v/>
@@ -4090,7 +4168,7 @@
         <v/>
       </c>
     </row>
-    <row r="120" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A120" s="35" t="str">
         <f t="shared" si="19"/>
         <v/>
@@ -4108,7 +4186,7 @@
         <v/>
       </c>
     </row>
-    <row r="121" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A121" s="35" t="str">
         <f t="shared" si="19"/>
         <v/>
@@ -4126,7 +4204,7 @@
         <v/>
       </c>
     </row>
-    <row r="122" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A122" s="35" t="str">
         <f t="shared" si="19"/>
         <v/>
@@ -4144,7 +4222,7 @@
         <v/>
       </c>
     </row>
-    <row r="123" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A123" s="35" t="str">
         <f t="shared" si="19"/>
         <v/>
@@ -4162,7 +4240,7 @@
         <v/>
       </c>
     </row>
-    <row r="124" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A124" s="35" t="str">
         <f t="shared" si="19"/>
         <v/>
@@ -4180,7 +4258,7 @@
         <v/>
       </c>
     </row>
-    <row r="125" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A125" s="35" t="str">
         <f t="shared" si="19"/>
         <v/>
@@ -4198,7 +4276,7 @@
         <v/>
       </c>
     </row>
-    <row r="126" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A126" s="35" t="str">
         <f t="shared" si="19"/>
         <v/>
@@ -4216,7 +4294,7 @@
         <v/>
       </c>
     </row>
-    <row r="127" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A127" s="35" t="str">
         <f t="shared" si="19"/>
         <v/>
@@ -4234,7 +4312,7 @@
         <v/>
       </c>
     </row>
-    <row r="128" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A128" s="35" t="str">
         <f t="shared" si="19"/>
         <v/>
@@ -4252,7 +4330,7 @@
         <v/>
       </c>
     </row>
-    <row r="129" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A129" s="35" t="str">
         <f t="shared" si="19"/>
         <v/>
@@ -4270,7 +4348,7 @@
         <v/>
       </c>
     </row>
-    <row r="130" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A130" s="35" t="str">
         <f t="shared" si="19"/>
         <v/>
@@ -4288,7 +4366,7 @@
         <v/>
       </c>
     </row>
-    <row r="131" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A131" s="35" t="str">
         <f t="shared" si="19"/>
         <v/>
@@ -4306,7 +4384,7 @@
         <v/>
       </c>
     </row>
-    <row r="132" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A132" s="35" t="str">
         <f t="shared" si="19"/>
         <v/>
@@ -4324,7 +4402,7 @@
         <v/>
       </c>
     </row>
-    <row r="133" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A133" s="35" t="str">
         <f t="shared" si="19"/>
         <v/>
@@ -4342,7 +4420,7 @@
         <v/>
       </c>
     </row>
-    <row r="134" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A134" s="35" t="str">
         <f t="shared" si="19"/>
         <v/>
@@ -4360,7 +4438,7 @@
         <v/>
       </c>
     </row>
-    <row r="135" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A135" s="35" t="str">
         <f t="shared" si="19"/>
         <v/>
@@ -4374,6 +4452,150 @@
         <v/>
       </c>
       <c r="G135" s="6" t="str">
+        <f t="shared" si="18"/>
+        <v/>
+      </c>
+    </row>
+    <row r="136" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A136" s="35" t="str">
+        <f t="shared" si="19"/>
+        <v/>
+      </c>
+      <c r="D136" s="6" t="str">
+        <f t="shared" si="20"/>
+        <v/>
+      </c>
+      <c r="E136" s="34" t="str">
+        <f t="shared" si="21"/>
+        <v/>
+      </c>
+      <c r="G136" s="6" t="str">
+        <f t="shared" si="18"/>
+        <v/>
+      </c>
+    </row>
+    <row r="137" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A137" s="35" t="str">
+        <f t="shared" si="19"/>
+        <v/>
+      </c>
+      <c r="D137" s="6" t="str">
+        <f t="shared" si="20"/>
+        <v/>
+      </c>
+      <c r="E137" s="34" t="str">
+        <f t="shared" si="21"/>
+        <v/>
+      </c>
+      <c r="G137" s="6" t="str">
+        <f t="shared" si="18"/>
+        <v/>
+      </c>
+    </row>
+    <row r="138" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A138" s="35" t="str">
+        <f t="shared" si="19"/>
+        <v/>
+      </c>
+      <c r="D138" s="6" t="str">
+        <f t="shared" si="20"/>
+        <v/>
+      </c>
+      <c r="E138" s="34" t="str">
+        <f t="shared" si="21"/>
+        <v/>
+      </c>
+      <c r="G138" s="6" t="str">
+        <f t="shared" si="18"/>
+        <v/>
+      </c>
+    </row>
+    <row r="139" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A139" s="35" t="str">
+        <f t="shared" si="19"/>
+        <v/>
+      </c>
+      <c r="D139" s="6" t="str">
+        <f t="shared" si="20"/>
+        <v/>
+      </c>
+      <c r="E139" s="34" t="str">
+        <f t="shared" si="21"/>
+        <v/>
+      </c>
+      <c r="G139" s="6" t="str">
+        <f t="shared" si="18"/>
+        <v/>
+      </c>
+    </row>
+    <row r="140" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A140" s="35" t="str">
+        <f t="shared" si="19"/>
+        <v/>
+      </c>
+      <c r="D140" s="6" t="str">
+        <f t="shared" si="20"/>
+        <v/>
+      </c>
+      <c r="E140" s="34" t="str">
+        <f t="shared" si="21"/>
+        <v/>
+      </c>
+      <c r="G140" s="6" t="str">
+        <f t="shared" si="18"/>
+        <v/>
+      </c>
+    </row>
+    <row r="141" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A141" s="35" t="str">
+        <f t="shared" si="19"/>
+        <v/>
+      </c>
+      <c r="D141" s="6" t="str">
+        <f t="shared" si="20"/>
+        <v/>
+      </c>
+      <c r="E141" s="34" t="str">
+        <f t="shared" si="21"/>
+        <v/>
+      </c>
+      <c r="G141" s="6" t="str">
+        <f t="shared" si="18"/>
+        <v/>
+      </c>
+    </row>
+    <row r="142" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A142" s="35" t="str">
+        <f t="shared" si="19"/>
+        <v/>
+      </c>
+      <c r="D142" s="6" t="str">
+        <f t="shared" si="20"/>
+        <v/>
+      </c>
+      <c r="E142" s="34" t="str">
+        <f t="shared" si="21"/>
+        <v/>
+      </c>
+      <c r="G142" s="6" t="str">
+        <f t="shared" si="18"/>
+        <v/>
+      </c>
+    </row>
+    <row r="143" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A143" s="35" t="str">
+        <f t="shared" si="19"/>
+        <v/>
+      </c>
+      <c r="D143" s="6" t="str">
+        <f t="shared" si="20"/>
+        <v/>
+      </c>
+      <c r="E143" s="34" t="str">
+        <f t="shared" si="21"/>
+        <v/>
+      </c>
+      <c r="G143" s="6" t="str">
         <f t="shared" si="18"/>
         <v/>
       </c>
@@ -4385,7 +4607,7 @@
     <mergeCell ref="E60:G60"/>
     <mergeCell ref="H4:H6"/>
     <mergeCell ref="D1:E1"/>
-    <mergeCell ref="A92:G92"/>
+    <mergeCell ref="A93:G93"/>
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="A7:A8"/>
@@ -4436,8 +4658,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G93:G1048576 G61:G77 G54:G56 G79 G81:G91 G5:G52">
-    <cfRule type="colorScale" priority="79">
+  <conditionalFormatting sqref="G94:G143 G62:G64 G54 G50:G52 G66:G77 G79 G81:G92 G9:G48">
+    <cfRule type="colorScale" priority="86">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -4448,8 +4670,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G93:G135 G62:G64 G54 G50:G52 G66:G77 G79 G81:G91 G9:G48">
-    <cfRule type="colorScale" priority="96">
+  <conditionalFormatting sqref="G94:G1048576 G61:G77 G54:G56 G79 G81:G92 G5:G52">
+    <cfRule type="colorScale" priority="79">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>

</xml_diff>

<commit_message>
Artifact Updated, Test Plan and Test Report Added
Requirements sheet also has ALL completion dates written and ready for submit.
</commit_message>
<xml_diff>
--- a/Documents/project requirements spreadsheet.xlsx
+++ b/Documents/project requirements spreadsheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/soapmac/Documents/GitHub/Shattered-Protocols-Text-RPG/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F1ACCF6-5CDD-024E-8012-AD2485FEB09F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F11B36A-0315-AA42-A276-5A54BAF9ED5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="160" yWindow="660" windowWidth="28480" windowHeight="15660" xr2:uid="{CAB5D44A-E176-404C-B398-BEAD2D9E6884}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="124">
   <si>
     <t>Intro to Software Engineering</t>
   </si>
@@ -403,6 +403,12 @@
   </si>
   <si>
     <t>Make level map</t>
+  </si>
+  <si>
+    <t>Iteration 4 plan report</t>
+  </si>
+  <si>
+    <t>Iteration 4 Test report</t>
   </si>
 </sst>
 </file>
@@ -897,6 +903,18 @@
     <xf numFmtId="14" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -926,18 +944,6 @@
     </xf>
     <xf numFmtId="14" fontId="12" fillId="6" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1295,17 +1301,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" s="22" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="76" t="s">
+      <c r="A1" s="80" t="s">
         <v>65</v>
       </c>
-      <c r="B1" s="77"/>
+      <c r="B1" s="81"/>
       <c r="C1" s="36" t="s">
         <v>10</v>
       </c>
-      <c r="D1" s="86" t="s">
+      <c r="D1" s="76" t="s">
         <v>31</v>
       </c>
-      <c r="E1" s="86"/>
+      <c r="E1" s="76"/>
       <c r="F1" s="37" t="s">
         <v>12</v>
       </c>
@@ -1315,10 +1321,10 @@
       <c r="H1" s="57"/>
     </row>
     <row r="2" spans="1:8" s="22" customFormat="1" ht="19" x14ac:dyDescent="0.2">
-      <c r="A2" s="78" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="79"/>
+      <c r="A2" s="82" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="83"/>
       <c r="C2" s="36" t="s">
         <v>11</v>
       </c>
@@ -1341,34 +1347,34 @@
     <row r="4" spans="1:8" s="7" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1"/>
       <c r="B4" s="2"/>
-      <c r="C4" s="83" t="s">
+      <c r="C4" s="87" t="s">
         <v>9</v>
       </c>
-      <c r="D4" s="83"/>
-      <c r="E4" s="83"/>
-      <c r="F4" s="83"/>
+      <c r="D4" s="87"/>
+      <c r="E4" s="87"/>
+      <c r="F4" s="87"/>
       <c r="G4" s="1"/>
-      <c r="H4" s="85" t="s">
+      <c r="H4" s="75" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="5" spans="1:8" s="7" customFormat="1" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="1"/>
       <c r="B5" s="2"/>
-      <c r="C5" s="82" t="s">
+      <c r="C5" s="86" t="s">
         <v>13</v>
       </c>
       <c r="D5" s="1"/>
-      <c r="E5" s="82" t="s">
+      <c r="E5" s="86" t="s">
         <v>44</v>
       </c>
-      <c r="F5" s="82" t="s">
+      <c r="F5" s="86" t="s">
         <v>45</v>
       </c>
-      <c r="G5" s="82" t="s">
+      <c r="G5" s="86" t="s">
         <v>46</v>
       </c>
-      <c r="H5" s="85"/>
+      <c r="H5" s="75"/>
     </row>
     <row r="6" spans="1:8" s="7" customFormat="1" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
@@ -1377,17 +1383,17 @@
       <c r="B6" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="C6" s="82"/>
+      <c r="C6" s="86"/>
       <c r="D6" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E6" s="82"/>
-      <c r="F6" s="82"/>
-      <c r="G6" s="82"/>
-      <c r="H6" s="85"/>
+      <c r="E6" s="86"/>
+      <c r="F6" s="86"/>
+      <c r="G6" s="86"/>
+      <c r="H6" s="75"/>
     </row>
     <row r="7" spans="1:8" s="48" customFormat="1" ht="52" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="80" t="s">
+      <c r="A7" s="84" t="s">
         <v>30</v>
       </c>
       <c r="B7" s="46"/>
@@ -1405,7 +1411,7 @@
       <c r="H7" s="60"/>
     </row>
     <row r="8" spans="1:8" s="3" customFormat="1" ht="61.5" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="81"/>
+      <c r="A8" s="85"/>
       <c r="B8" s="8"/>
       <c r="C8" s="10"/>
       <c r="D8" s="10" t="s">
@@ -1485,9 +1491,9 @@
       <c r="E11" s="11">
         <v>45628</v>
       </c>
-      <c r="F11" s="11" t="str">
+      <c r="F11" s="11">
         <f>IF(F95&gt;0,F95,"")</f>
-        <v/>
+        <v>45628</v>
       </c>
       <c r="G11" s="6">
         <f>IF(AND(E11&gt;0,ISNUMBER(F11)),F11-E11,0)</f>
@@ -1512,7 +1518,7 @@
         <v>45628</v>
       </c>
       <c r="F12" s="11">
-        <f t="shared" ref="F12:F19" si="1">IF(F96&gt;0,F96,"")</f>
+        <f t="shared" ref="F12:F13" si="1">IF(F96&gt;0,F96,"")</f>
         <v>45628</v>
       </c>
       <c r="G12" s="6">
@@ -1564,7 +1570,7 @@
         <v>45628</v>
       </c>
       <c r="F14" s="11">
-        <f t="shared" si="1"/>
+        <f>IF(F98&gt;0,F98,"")</f>
         <v>45628</v>
       </c>
       <c r="G14" s="6">
@@ -1590,7 +1596,7 @@
         <v>45628</v>
       </c>
       <c r="F15" s="11">
-        <f t="shared" si="1"/>
+        <f>IF(F99&gt;0,F99,"")</f>
         <v>45628</v>
       </c>
       <c r="G15" s="6">
@@ -1616,7 +1622,7 @@
         <v>45628</v>
       </c>
       <c r="F16" s="11">
-        <f t="shared" si="1"/>
+        <f>IF(F100&gt;0,F100,"")</f>
         <v>45628</v>
       </c>
       <c r="G16" s="6">
@@ -1642,7 +1648,7 @@
         <v>45628</v>
       </c>
       <c r="F17" s="11">
-        <f t="shared" si="1"/>
+        <f>IF(F101&gt;0,F101,"")</f>
         <v>45607</v>
       </c>
       <c r="G17" s="6">
@@ -1668,7 +1674,7 @@
         <v>45628</v>
       </c>
       <c r="F18" s="11">
-        <f t="shared" si="1"/>
+        <f>IF(F102&gt;0,F102,"")</f>
         <v>45628</v>
       </c>
       <c r="G18" s="6">
@@ -1693,9 +1699,9 @@
       <c r="E19" s="11">
         <v>45628</v>
       </c>
-      <c r="F19" s="11" t="str">
-        <f t="shared" si="1"/>
-        <v/>
+      <c r="F19" s="11">
+        <f>IF(F103&gt;0,F103,"")</f>
+        <v>45628</v>
       </c>
       <c r="G19" s="6">
         <f t="shared" si="2"/>
@@ -1955,7 +1961,7 @@
         <f t="shared" si="3"/>
         <v>-20</v>
       </c>
-      <c r="H29" s="87" t="s">
+      <c r="H29" s="77" t="s">
         <v>112</v>
       </c>
     </row>
@@ -1983,7 +1989,7 @@
         <f t="shared" si="3"/>
         <v>-20</v>
       </c>
-      <c r="H30" s="88"/>
+      <c r="H30" s="78"/>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A31" s="43">
@@ -2009,7 +2015,7 @@
         <f t="shared" si="3"/>
         <v>-20</v>
       </c>
-      <c r="H31" s="88"/>
+      <c r="H31" s="78"/>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A32" s="43">
@@ -2035,7 +2041,7 @@
         <f t="shared" si="3"/>
         <v>-20</v>
       </c>
-      <c r="H32" s="88"/>
+      <c r="H32" s="78"/>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A33" s="43">
@@ -2061,7 +2067,7 @@
         <f t="shared" si="3"/>
         <v>-20</v>
       </c>
-      <c r="H33" s="88"/>
+      <c r="H33" s="78"/>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A34" s="43">
@@ -2572,11 +2578,11 @@
         <f t="shared" ref="D53:D106" si="7">IF(B53="","",D52)</f>
         <v>2</v>
       </c>
-      <c r="E53" s="84" t="s">
+      <c r="E53" s="88" t="s">
         <v>81</v>
       </c>
-      <c r="F53" s="84"/>
-      <c r="G53" s="84"/>
+      <c r="F53" s="88"/>
+      <c r="G53" s="88"/>
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A54" s="35">
@@ -2670,11 +2676,11 @@
       <c r="D57" s="6">
         <v>2</v>
       </c>
-      <c r="E57" s="84" t="s">
+      <c r="E57" s="88" t="s">
         <v>58</v>
       </c>
-      <c r="F57" s="84"/>
-      <c r="G57" s="84"/>
+      <c r="F57" s="88"/>
+      <c r="G57" s="88"/>
       <c r="H57" s="63" t="s">
         <v>116</v>
       </c>
@@ -2694,11 +2700,11 @@
         <f>IF(B58="","",D56)</f>
         <v>2</v>
       </c>
-      <c r="E58" s="84" t="s">
+      <c r="E58" s="88" t="s">
         <v>58</v>
       </c>
-      <c r="F58" s="84"/>
-      <c r="G58" s="84"/>
+      <c r="F58" s="88"/>
+      <c r="G58" s="88"/>
       <c r="H58" s="63" t="s">
         <v>116</v>
       </c>
@@ -2718,11 +2724,11 @@
         <f>IF(B59="","",D54)</f>
         <v>2</v>
       </c>
-      <c r="E59" s="84" t="s">
+      <c r="E59" s="88" t="s">
         <v>58</v>
       </c>
-      <c r="F59" s="84"/>
-      <c r="G59" s="84"/>
+      <c r="F59" s="88"/>
+      <c r="G59" s="88"/>
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A60" s="35">
@@ -2739,11 +2745,11 @@
         <f>IF(B60="","",D59)</f>
         <v>2</v>
       </c>
-      <c r="E60" s="84" t="s">
+      <c r="E60" s="88" t="s">
         <v>81</v>
       </c>
-      <c r="F60" s="84"/>
-      <c r="G60" s="84"/>
+      <c r="F60" s="88"/>
+      <c r="G60" s="88"/>
       <c r="H60" s="63" t="s">
         <v>117</v>
       </c>
@@ -2936,7 +2942,7 @@
     </row>
     <row r="68" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A68" s="35">
-        <f t="shared" ref="A68:A106" si="16">IF(B68="","",IF(D68=D67,A67+1,(D68*100)))</f>
+        <f t="shared" ref="A68:A97" si="16">IF(B68="","",IF(D68=D67,A67+1,(D68*100)))</f>
         <v>302</v>
       </c>
       <c r="B68" s="5" t="s">
@@ -3205,11 +3211,11 @@
         <f t="shared" si="7"/>
         <v>3</v>
       </c>
-      <c r="E78" s="84" t="s">
+      <c r="E78" s="88" t="s">
         <v>81</v>
       </c>
-      <c r="F78" s="84"/>
-      <c r="G78" s="84"/>
+      <c r="F78" s="88"/>
+      <c r="G78" s="88"/>
       <c r="H78" s="63" t="s">
         <v>119</v>
       </c>
@@ -3254,11 +3260,11 @@
       <c r="D80" s="6">
         <v>3</v>
       </c>
-      <c r="E80" s="84" t="s">
+      <c r="E80" s="88" t="s">
         <v>81</v>
       </c>
-      <c r="F80" s="84"/>
-      <c r="G80" s="84"/>
+      <c r="F80" s="88"/>
+      <c r="G80" s="88"/>
     </row>
     <row r="81" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A81" s="35">
@@ -3356,9 +3362,12 @@
       <c r="E84" s="34">
         <v>45625</v>
       </c>
+      <c r="F84" s="11">
+        <v>45628</v>
+      </c>
       <c r="G84" s="6">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="85" spans="1:8" ht="17" x14ac:dyDescent="0.2">
@@ -3568,15 +3577,15 @@
       </c>
     </row>
     <row r="93" spans="1:8" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A93" s="75" t="s">
+      <c r="A93" s="79" t="s">
         <v>110</v>
       </c>
-      <c r="B93" s="75"/>
-      <c r="C93" s="75"/>
-      <c r="D93" s="75"/>
-      <c r="E93" s="75"/>
-      <c r="F93" s="75"/>
-      <c r="G93" s="75"/>
+      <c r="B93" s="79"/>
+      <c r="C93" s="79"/>
+      <c r="D93" s="79"/>
+      <c r="E93" s="79"/>
+      <c r="F93" s="79"/>
+      <c r="G93" s="79"/>
     </row>
     <row r="94" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A94" s="35">
@@ -3622,6 +3631,9 @@
       <c r="E95" s="34">
         <v>45628</v>
       </c>
+      <c r="F95" s="11">
+        <v>45628</v>
+      </c>
       <c r="G95" s="6">
         <f t="shared" ref="G95:G143" si="18">IF(B95="","",IF(AND(E95&gt;0,F95&gt;0),F95-E95,0))</f>
         <v>0</v>
@@ -3681,7 +3693,7 @@
     </row>
     <row r="98" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A98" s="35">
-        <f t="shared" si="16"/>
+        <f>IF(B98="","",IF(D98=D97,A97+1,(D98*100)))</f>
         <v>414</v>
       </c>
       <c r="B98" s="5" t="s">
@@ -3691,7 +3703,7 @@
         <v>34</v>
       </c>
       <c r="D98" s="6">
-        <f t="shared" si="7"/>
+        <f>IF(B98="","",D97)</f>
         <v>4</v>
       </c>
       <c r="E98" s="34">
@@ -3707,7 +3719,7 @@
     </row>
     <row r="99" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A99" s="35">
-        <f t="shared" si="16"/>
+        <f>IF(B99="","",IF(D99=D98,A98+1,(D99*100)))</f>
         <v>415</v>
       </c>
       <c r="B99" s="5" t="s">
@@ -3733,7 +3745,7 @@
     </row>
     <row r="100" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A100" s="35">
-        <f t="shared" si="16"/>
+        <f>IF(B100="","",IF(D100=D99,A99+1,(D100*100)))</f>
         <v>416</v>
       </c>
       <c r="B100" s="5" t="s">
@@ -3759,7 +3771,7 @@
     </row>
     <row r="101" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A101" s="35">
-        <f t="shared" si="16"/>
+        <f>IF(B101="","",IF(D101=D100,A100+1,(D101*100)))</f>
         <v>417</v>
       </c>
       <c r="B101" s="5" t="s">
@@ -3786,7 +3798,7 @@
     </row>
     <row r="102" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A102" s="35">
-        <f t="shared" si="16"/>
+        <f>IF(B102="","",IF(D102=D101,A101+1,(D102*100)))</f>
         <v>418</v>
       </c>
       <c r="B102" s="5" t="s">
@@ -3812,7 +3824,7 @@
     </row>
     <row r="103" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A103" s="35">
-        <f t="shared" si="16"/>
+        <f>IF(B103="","",IF(D103=D102,A102+1,(D103*100)))</f>
         <v>419</v>
       </c>
       <c r="B103" s="5" t="s">
@@ -3828,6 +3840,9 @@
       <c r="E103" s="34">
         <v>45628</v>
       </c>
+      <c r="F103" s="11">
+        <v>45628</v>
+      </c>
       <c r="G103" s="6">
         <f t="shared" si="18"/>
         <v>0</v>
@@ -3835,7 +3850,7 @@
     </row>
     <row r="104" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A104" s="35">
-        <f t="shared" si="16"/>
+        <f>IF(B104="","",IF(D104=D103,A103+1,(D104*100)))</f>
         <v>420</v>
       </c>
       <c r="B104" s="72" t="s">
@@ -3861,7 +3876,7 @@
     </row>
     <row r="105" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A105" s="35">
-        <f t="shared" si="16"/>
+        <f>IF(B105="","",IF(D105=D104,A104+1,(D105*100)))</f>
         <v>421</v>
       </c>
       <c r="B105" s="5" t="s">
@@ -3887,7 +3902,7 @@
     </row>
     <row r="106" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A106" s="35">
-        <f t="shared" si="16"/>
+        <f>IF(B106="","",IF(D106=D105,A105+1,(D106*100)))</f>
         <v>422</v>
       </c>
       <c r="B106" s="5" t="s">
@@ -3912,52 +3927,68 @@
       </c>
     </row>
     <row r="107" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A107" s="35" t="str">
-        <f>IF(B107="","",IF(D107=#REF!,#REF!+1,(D107*100)))</f>
-        <v/>
-      </c>
-      <c r="D107" s="6" t="str">
-        <f>IF(B107="","",#REF!)</f>
-        <v/>
-      </c>
-      <c r="E107" s="34" t="str">
-        <f>IF(B107="","",IF(D107=#REF!,#REF!,#REF!+14))</f>
-        <v/>
-      </c>
-      <c r="G107" s="6" t="str">
-        <f t="shared" si="18"/>
-        <v/>
+      <c r="A107" s="35">
+        <f>IF(B107="","",IF(D107=D106,A106+1,(D107*100)))</f>
+        <v>423</v>
+      </c>
+      <c r="B107" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="C107" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="D107" s="6">
+        <f>IF(B107="","",D106)</f>
+        <v>4</v>
+      </c>
+      <c r="E107" s="34">
+        <v>45628</v>
+      </c>
+      <c r="F107" s="11">
+        <v>45628</v>
+      </c>
+      <c r="G107" s="6">
+        <f t="shared" ref="G107:G108" si="19">IF(B107="","",IF(AND(E107&gt;0,F107&gt;0),F107-E107,0))</f>
+        <v>0</v>
       </c>
     </row>
     <row r="108" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A108" s="35" t="str">
-        <f t="shared" ref="A108:A143" si="19">IF(B108="","",IF(D108=D107,A107+1,(D108*100)))</f>
-        <v/>
-      </c>
-      <c r="D108" s="6" t="str">
-        <f t="shared" ref="D108:D143" si="20">IF(B108="","",D107)</f>
-        <v/>
-      </c>
-      <c r="E108" s="34" t="str">
-        <f t="shared" ref="E108:E143" si="21">IF(B108="","",IF(D108=D107,E107,E107+14))</f>
-        <v/>
-      </c>
-      <c r="G108" s="6" t="str">
-        <f t="shared" si="18"/>
-        <v/>
+      <c r="A108" s="35">
+        <f>IF(B108="","",IF(D108=D107,A107+1,(D108*100)))</f>
+        <v>424</v>
+      </c>
+      <c r="B108" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="C108" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="D108" s="6">
+        <f>IF(B108="","",D107)</f>
+        <v>4</v>
+      </c>
+      <c r="E108" s="34">
+        <v>45628</v>
+      </c>
+      <c r="F108" s="11">
+        <v>45628</v>
+      </c>
+      <c r="G108" s="6">
+        <f t="shared" si="19"/>
+        <v>0</v>
       </c>
     </row>
     <row r="109" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A109" s="35" t="str">
-        <f t="shared" si="19"/>
+        <f>IF(B109="","",IF(D109=D108,A108+1,(D109*100)))</f>
         <v/>
       </c>
       <c r="D109" s="6" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" ref="D108:D143" si="20">IF(B109="","",D108)</f>
         <v/>
       </c>
       <c r="E109" s="34" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" ref="E108:E143" si="21">IF(B109="","",IF(D109=D108,E108,E108+14))</f>
         <v/>
       </c>
       <c r="G109" s="6" t="str">
@@ -3967,7 +3998,7 @@
     </row>
     <row r="110" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A110" s="35" t="str">
-        <f t="shared" si="19"/>
+        <f>IF(B110="","",IF(D110=D109,A109+1,(D110*100)))</f>
         <v/>
       </c>
       <c r="D110" s="6" t="str">
@@ -3985,7 +4016,7 @@
     </row>
     <row r="111" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A111" s="35" t="str">
-        <f t="shared" si="19"/>
+        <f>IF(B111="","",IF(D111=D110,A110+1,(D111*100)))</f>
         <v/>
       </c>
       <c r="D111" s="6" t="str">
@@ -4003,7 +4034,7 @@
     </row>
     <row r="112" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A112" s="35" t="str">
-        <f t="shared" si="19"/>
+        <f>IF(B112="","",IF(D112=D111,A111+1,(D112*100)))</f>
         <v/>
       </c>
       <c r="D112" s="6" t="str">
@@ -4021,7 +4052,7 @@
     </row>
     <row r="113" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A113" s="35" t="str">
-        <f t="shared" si="19"/>
+        <f>IF(B113="","",IF(D113=D112,A112+1,(D113*100)))</f>
         <v/>
       </c>
       <c r="D113" s="6" t="str">
@@ -4039,7 +4070,7 @@
     </row>
     <row r="114" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A114" s="35" t="str">
-        <f t="shared" si="19"/>
+        <f>IF(B114="","",IF(D114=D113,A113+1,(D114*100)))</f>
         <v/>
       </c>
       <c r="D114" s="6" t="str">
@@ -4057,7 +4088,7 @@
     </row>
     <row r="115" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A115" s="35" t="str">
-        <f t="shared" si="19"/>
+        <f>IF(B115="","",IF(D115=D114,A114+1,(D115*100)))</f>
         <v/>
       </c>
       <c r="D115" s="6" t="str">
@@ -4075,7 +4106,7 @@
     </row>
     <row r="116" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A116" s="35" t="str">
-        <f t="shared" si="19"/>
+        <f>IF(B116="","",IF(D116=D115,A115+1,(D116*100)))</f>
         <v/>
       </c>
       <c r="D116" s="6" t="str">
@@ -4093,7 +4124,7 @@
     </row>
     <row r="117" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A117" s="35" t="str">
-        <f t="shared" si="19"/>
+        <f>IF(B117="","",IF(D117=D116,A116+1,(D117*100)))</f>
         <v/>
       </c>
       <c r="D117" s="6" t="str">
@@ -4111,7 +4142,7 @@
     </row>
     <row r="118" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A118" s="35" t="str">
-        <f t="shared" si="19"/>
+        <f>IF(B118="","",IF(D118=D117,A117+1,(D118*100)))</f>
         <v/>
       </c>
       <c r="D118" s="6" t="str">
@@ -4129,7 +4160,7 @@
     </row>
     <row r="119" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A119" s="35" t="str">
-        <f t="shared" si="19"/>
+        <f>IF(B119="","",IF(D119=D118,A118+1,(D119*100)))</f>
         <v/>
       </c>
       <c r="D119" s="6" t="str">
@@ -4147,7 +4178,7 @@
     </row>
     <row r="120" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A120" s="35" t="str">
-        <f t="shared" si="19"/>
+        <f>IF(B120="","",IF(D120=D119,A119+1,(D120*100)))</f>
         <v/>
       </c>
       <c r="D120" s="6" t="str">
@@ -4165,7 +4196,7 @@
     </row>
     <row r="121" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A121" s="35" t="str">
-        <f t="shared" si="19"/>
+        <f>IF(B121="","",IF(D121=D120,A120+1,(D121*100)))</f>
         <v/>
       </c>
       <c r="D121" s="6" t="str">
@@ -4183,7 +4214,7 @@
     </row>
     <row r="122" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A122" s="35" t="str">
-        <f t="shared" si="19"/>
+        <f>IF(B122="","",IF(D122=D121,A121+1,(D122*100)))</f>
         <v/>
       </c>
       <c r="D122" s="6" t="str">
@@ -4201,7 +4232,7 @@
     </row>
     <row r="123" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A123" s="35" t="str">
-        <f t="shared" si="19"/>
+        <f>IF(B123="","",IF(D123=D122,A122+1,(D123*100)))</f>
         <v/>
       </c>
       <c r="D123" s="6" t="str">
@@ -4219,7 +4250,7 @@
     </row>
     <row r="124" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A124" s="35" t="str">
-        <f t="shared" si="19"/>
+        <f>IF(B124="","",IF(D124=D123,A123+1,(D124*100)))</f>
         <v/>
       </c>
       <c r="D124" s="6" t="str">
@@ -4237,7 +4268,7 @@
     </row>
     <row r="125" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A125" s="35" t="str">
-        <f t="shared" si="19"/>
+        <f>IF(B125="","",IF(D125=D124,A124+1,(D125*100)))</f>
         <v/>
       </c>
       <c r="D125" s="6" t="str">
@@ -4255,7 +4286,7 @@
     </row>
     <row r="126" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A126" s="35" t="str">
-        <f t="shared" si="19"/>
+        <f>IF(B126="","",IF(D126=D125,A125+1,(D126*100)))</f>
         <v/>
       </c>
       <c r="D126" s="6" t="str">
@@ -4273,7 +4304,7 @@
     </row>
     <row r="127" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A127" s="35" t="str">
-        <f t="shared" si="19"/>
+        <f>IF(B127="","",IF(D127=D126,A126+1,(D127*100)))</f>
         <v/>
       </c>
       <c r="D127" s="6" t="str">
@@ -4291,7 +4322,7 @@
     </row>
     <row r="128" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A128" s="35" t="str">
-        <f t="shared" si="19"/>
+        <f>IF(B128="","",IF(D128=D127,A127+1,(D128*100)))</f>
         <v/>
       </c>
       <c r="D128" s="6" t="str">
@@ -4309,7 +4340,7 @@
     </row>
     <row r="129" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A129" s="35" t="str">
-        <f t="shared" si="19"/>
+        <f>IF(B129="","",IF(D129=D128,A128+1,(D129*100)))</f>
         <v/>
       </c>
       <c r="D129" s="6" t="str">
@@ -4327,7 +4358,7 @@
     </row>
     <row r="130" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A130" s="35" t="str">
-        <f t="shared" si="19"/>
+        <f>IF(B130="","",IF(D130=D129,A129+1,(D130*100)))</f>
         <v/>
       </c>
       <c r="D130" s="6" t="str">
@@ -4345,7 +4376,7 @@
     </row>
     <row r="131" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A131" s="35" t="str">
-        <f t="shared" si="19"/>
+        <f>IF(B131="","",IF(D131=D130,A130+1,(D131*100)))</f>
         <v/>
       </c>
       <c r="D131" s="6" t="str">
@@ -4363,7 +4394,7 @@
     </row>
     <row r="132" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A132" s="35" t="str">
-        <f t="shared" si="19"/>
+        <f>IF(B132="","",IF(D132=D131,A131+1,(D132*100)))</f>
         <v/>
       </c>
       <c r="D132" s="6" t="str">
@@ -4381,7 +4412,7 @@
     </row>
     <row r="133" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A133" s="35" t="str">
-        <f t="shared" si="19"/>
+        <f>IF(B133="","",IF(D133=D132,A132+1,(D133*100)))</f>
         <v/>
       </c>
       <c r="D133" s="6" t="str">
@@ -4399,7 +4430,7 @@
     </row>
     <row r="134" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A134" s="35" t="str">
-        <f t="shared" si="19"/>
+        <f>IF(B134="","",IF(D134=D133,A133+1,(D134*100)))</f>
         <v/>
       </c>
       <c r="D134" s="6" t="str">
@@ -4417,7 +4448,7 @@
     </row>
     <row r="135" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A135" s="35" t="str">
-        <f t="shared" si="19"/>
+        <f>IF(B135="","",IF(D135=D134,A134+1,(D135*100)))</f>
         <v/>
       </c>
       <c r="D135" s="6" t="str">
@@ -4435,7 +4466,7 @@
     </row>
     <row r="136" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A136" s="35" t="str">
-        <f t="shared" si="19"/>
+        <f>IF(B136="","",IF(D136=D135,A135+1,(D136*100)))</f>
         <v/>
       </c>
       <c r="D136" s="6" t="str">
@@ -4453,7 +4484,7 @@
     </row>
     <row r="137" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A137" s="35" t="str">
-        <f t="shared" si="19"/>
+        <f>IF(B137="","",IF(D137=D136,A136+1,(D137*100)))</f>
         <v/>
       </c>
       <c r="D137" s="6" t="str">
@@ -4471,7 +4502,7 @@
     </row>
     <row r="138" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A138" s="35" t="str">
-        <f t="shared" si="19"/>
+        <f>IF(B138="","",IF(D138=D137,A137+1,(D138*100)))</f>
         <v/>
       </c>
       <c r="D138" s="6" t="str">
@@ -4489,7 +4520,7 @@
     </row>
     <row r="139" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A139" s="35" t="str">
-        <f t="shared" si="19"/>
+        <f>IF(B139="","",IF(D139=D138,A138+1,(D139*100)))</f>
         <v/>
       </c>
       <c r="D139" s="6" t="str">
@@ -4507,7 +4538,7 @@
     </row>
     <row r="140" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A140" s="35" t="str">
-        <f t="shared" si="19"/>
+        <f>IF(B140="","",IF(D140=D139,A139+1,(D140*100)))</f>
         <v/>
       </c>
       <c r="D140" s="6" t="str">
@@ -4525,7 +4556,7 @@
     </row>
     <row r="141" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A141" s="35" t="str">
-        <f t="shared" si="19"/>
+        <f>IF(B141="","",IF(D141=D140,A140+1,(D141*100)))</f>
         <v/>
       </c>
       <c r="D141" s="6" t="str">
@@ -4543,7 +4574,7 @@
     </row>
     <row r="142" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A142" s="35" t="str">
-        <f t="shared" si="19"/>
+        <f>IF(B142="","",IF(D142=D141,A141+1,(D142*100)))</f>
         <v/>
       </c>
       <c r="D142" s="6" t="str">
@@ -4561,7 +4592,7 @@
     </row>
     <row r="143" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A143" s="35" t="str">
-        <f t="shared" si="19"/>
+        <f>IF(B143="","",IF(D143=D142,A142+1,(D143*100)))</f>
         <v/>
       </c>
       <c r="D143" s="6" t="str">
@@ -4579,6 +4610,9 @@
     </row>
   </sheetData>
   <mergeCells count="19">
+    <mergeCell ref="E53:G53"/>
+    <mergeCell ref="E78:G78"/>
+    <mergeCell ref="E60:G60"/>
     <mergeCell ref="H4:H6"/>
     <mergeCell ref="D1:E1"/>
     <mergeCell ref="H29:H33"/>
@@ -4595,9 +4629,6 @@
     <mergeCell ref="E57:G57"/>
     <mergeCell ref="E58:G58"/>
     <mergeCell ref="E59:G59"/>
-    <mergeCell ref="E53:G53"/>
-    <mergeCell ref="E78:G78"/>
-    <mergeCell ref="E60:G60"/>
   </mergeCells>
   <conditionalFormatting sqref="G49">
     <cfRule type="colorScale" priority="8">
@@ -4635,7 +4666,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G94:G143 G62:G64 G54 G50:G52 G66:G77 G79 G81:G92 G9:G48">
+  <conditionalFormatting sqref="G62:G64 G54 G50:G52 G66:G77 G79 G81:G92 G9:G48 G94:G143">
     <cfRule type="colorScale" priority="86">
       <colorScale>
         <cfvo type="min"/>
@@ -4647,7 +4678,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G94:G1048576 G61:G77 G54:G56 G79 G81:G92 G5:G52">
+  <conditionalFormatting sqref="G61:G77 G54:G56 G79 G81:G92 G5:G52 G94:G1048576">
     <cfRule type="colorScale" priority="79">
       <colorScale>
         <cfvo type="min"/>

</xml_diff>